<commit_message>
docs: richte IPA-Kontext auf Cortex-Cloud-Projekt aus
- Master-Rule auf die reale IPA-Aufgabenstellung (Cortex Cloud) angepasst, Shift-Planning-Reste entfernt
- .gitignore um /contextwindow ergaenzt
- Zeitplan: Bild Zeitplan.png via figure-Shortcode eingebunden
- Arbeitsplatz: Platzhalter fuer fehlendes Bild markiert
- Excel-Zeitplan aktualisiert

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/IPA_Zeitplan_Nicola_Maeder.xlsx
+++ b/IPA_Zeitplan_Nicola_Maeder.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\taamanii\Documents\Individuelle Praktische Arbeit Nicola\individuelle-praktische-arbeit-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8B6B5C4-84BA-4C51-B86F-56CA60715ECB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A327F332-557B-489B-BEA6-2F23E1117D26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{09F15F46-AED7-3C4E-9C62-04C59C5DDA6F}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="68">
   <si>
     <t>Tag</t>
   </si>
@@ -225,9 +225,6 @@
     <t>Aussehen des Webinterfaces &amp; des PDF Reporting</t>
   </si>
   <si>
-    <t>Projektmanagementmethoden</t>
-  </si>
-  <si>
     <t>Kurzfassung schreiben</t>
   </si>
   <si>
@@ -263,6 +260,12 @@
   <si>
     <t>ZEITPLAN Nicola Maeder 22.4.2026</t>
   </si>
+  <si>
+    <t>Projektmanagementmethoden, Arbeitsorganisation</t>
+  </si>
+  <si>
+    <t>F+A6:D86ALSCH</t>
+  </si>
 </sst>
 </file>
 
@@ -272,9 +275,16 @@
     <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -793,69 +803,69 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="286">
+  <cellXfs count="289">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="15" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -863,38 +873,14 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="4" borderId="11" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="4" borderId="11" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
     </xf>
     <xf numFmtId="2" fontId="7" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
@@ -911,166 +897,190 @@
     <xf numFmtId="2" fontId="7" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="26" borderId="2" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="26" borderId="16" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="28" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="28" borderId="11" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="26" borderId="2" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="26" borderId="16" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="28" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="28" borderId="11" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="28" borderId="11" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="28" borderId="11" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="31" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="29" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="30" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="20" fontId="3" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="2" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="20" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="32" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="32" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="32" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="32" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="6" fillId="29" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="32" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="7" fillId="29" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="29" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="29" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="20" fontId="4" fillId="4" borderId="13" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="5" fillId="4" borderId="13" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="20" fontId="4" fillId="4" borderId="14" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="5" fillId="4" borderId="14" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="20" fontId="4" fillId="4" borderId="15" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="20" fontId="5" fillId="4" borderId="15" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1078,7 +1088,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1086,40 +1096,37 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="180" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="180" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="180" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1127,34 +1134,34 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="20" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="20" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="20" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="20" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="6" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="6" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="6" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="6" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="6" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="6" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="6" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="6" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="6" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="6" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="6" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="6" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1162,7 +1169,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1170,13 +1177,13 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1184,7 +1191,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1192,43 +1199,43 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="6" borderId="2" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="6" borderId="2" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="6" borderId="6" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="6" borderId="6" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="6" borderId="5" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="6" borderId="5" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="6" borderId="9" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="6" borderId="9" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="8" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="8" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="8" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="8" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="8" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="8" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="8" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="8" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="8" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="8" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1236,7 +1243,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1244,13 +1251,13 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="19" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="19" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1258,16 +1265,13 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="19" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="19" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1275,7 +1279,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1283,25 +1287,25 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="8" borderId="2" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="8" borderId="2" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="8" borderId="6" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="8" borderId="6" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="8" borderId="5" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="8" borderId="18" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="8" borderId="18" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1309,7 +1313,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1317,43 +1321,43 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="11" borderId="2" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="11" borderId="2" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="11" borderId="6" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="11" borderId="6" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="11" borderId="5" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="11" borderId="5" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="11" borderId="9" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="11" borderId="9" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="11" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="11" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="11" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="11" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="11" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="11" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="11" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="11" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="11" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="11" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="11" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="11" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1361,10 +1365,10 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1372,7 +1376,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1380,13 +1384,13 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="19" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="19" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1394,10 +1398,10 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1405,7 +1409,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1413,40 +1417,40 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="14" borderId="2" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="14" borderId="2" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="14" borderId="16" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="14" borderId="16" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="14" borderId="6" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="14" borderId="6" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="14" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="14" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="14" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="14" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="14" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="14" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="14" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="14" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="14" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="14" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="14" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="14" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1454,7 +1458,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1462,40 +1466,40 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="17" borderId="2" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="17" borderId="2" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="17" borderId="16" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="17" borderId="16" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="17" borderId="6" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="17" borderId="6" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="17" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="17" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="17" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="17" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="17" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="17" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="17" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="17" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="17" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="17" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="17" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="17" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1503,7 +1507,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1511,13 +1515,13 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="19" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="19" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1525,10 +1529,10 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1536,7 +1540,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1544,13 +1548,13 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="19" borderId="19" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="19" borderId="19" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1558,34 +1562,34 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="19" borderId="19" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="19" borderId="19" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="19" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="20" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="20" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="20" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="20" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="20" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="20" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="20" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="20" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="20" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="20" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="20" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="20" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="21" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1593,7 +1597,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="21" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1601,13 +1605,13 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="22" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="22" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="22" borderId="19" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="22" borderId="19" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1615,7 +1619,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="20" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1623,22 +1627,22 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="20" borderId="2" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="20" borderId="2" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="20" borderId="16" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="20" borderId="16" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="20" borderId="6" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="20" borderId="6" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="23" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="23" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1646,7 +1650,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="23" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="23" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1654,34 +1658,34 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="6" borderId="16" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="6" borderId="16" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="6" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="6" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="6" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="6" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="6" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="6" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="6" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="6" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="6" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="6" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="6" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="6" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="21" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1689,13 +1693,13 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="22" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="22" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="22" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="22" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="21" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1703,13 +1707,13 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="22" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="22" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1717,7 +1721,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1725,13 +1729,13 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="24" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="19" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="24" borderId="19" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1739,10 +1743,10 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="24" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -1750,88 +1754,103 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="24" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="25" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="25" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="25" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="25" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="25" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="25" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="25" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="25" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="25" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="25" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="25" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="25" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="27" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="27" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="27" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="27" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="28" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="28" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="28" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="28" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="24" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="24" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="25" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="25" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="25" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="25" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="25" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="25" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="25" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="25" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="25" borderId="2" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="25" borderId="2" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="25" borderId="16" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="25" borderId="16" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="25" borderId="5" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="25" borderId="5" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="25" borderId="18" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="25" borderId="18" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="32" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="32" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="26" borderId="6" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="26" borderId="20" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="27" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="26" borderId="6" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="26" borderId="20" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="27" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="27" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="27" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="29" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="29" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="29" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="23" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2202,8 +2221,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:54" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="107" t="s">
-        <v>66</v>
+      <c r="A1" s="288" t="s">
+        <v>65</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -2286,7 +2305,7 @@
       <c r="BB1" s="86"/>
     </row>
     <row r="2" spans="1:54" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A2" s="108"/>
+      <c r="A2" s="107"/>
       <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
@@ -2366,7 +2385,7 @@
       <c r="BB2" s="92"/>
     </row>
     <row r="3" spans="1:54" ht="83.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A3" s="108"/>
+      <c r="A3" s="107"/>
       <c r="B3" s="4" t="s">
         <v>3</v>
       </c>
@@ -2528,7 +2547,7 @@
       </c>
     </row>
     <row r="4" spans="1:54" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A4" s="109"/>
+      <c r="A4" s="108"/>
       <c r="B4" s="7" t="s">
         <v>10</v>
       </c>
@@ -2557,11 +2576,11 @@
       </c>
       <c r="K4" s="9" cm="1">
         <f t="array" ref="K4">_xlfn.LET(_xlpm.r, K7:K90,SUM( _xlfn._xlws.FILTER( _xlpm.r, MOD(ROW(_xlpm.r) - ROW(INDEX(_xlpm.r,1,1)) + 1, 2) = 0 ) ))</f>
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="L4" s="10" cm="1">
         <f t="array" ref="L4">_xlfn.LET(_xlpm.r, L7:L90,SUM( _xlfn._xlws.FILTER( _xlpm.r, MOD(ROW(_xlpm.r) - ROW(INDEX(_xlpm.r,1,1)) + 1, 2) = 0 ) ))</f>
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="M4" s="10" cm="1">
         <f t="array" ref="M4">_xlfn.LET(_xlpm.r, M7:M92,SUM( _xlfn._xlws.FILTER( _xlpm.r, MOD(ROW(_xlpm.r) - ROW(INDEX(_xlpm.r,1,1)) + 1, 2) = 0 ) ))</f>
@@ -2796,7 +2815,7 @@
       </c>
       <c r="S5" s="10" cm="1">
         <f t="array" ref="S5">_xlfn.LET(_xlpm.r, S8:S92,SUM( _xlfn._xlws.FILTER( _xlpm.r, MOD(ROW(_xlpm.r) - ROW(INDEX(_xlpm.r,1,1)) + 1, 2) = 0 ) ))</f>
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="T5" s="11" cm="1">
         <f t="array" ref="T5">_xlfn.LET(_xlpm.r, T8:T92,SUM( _xlfn._xlws.FILTER( _xlpm.r, MOD(ROW(_xlpm.r) - ROW(INDEX(_xlpm.r,1,1)) + 1, 2) = 0 ) ))</f>
@@ -2892,7 +2911,7 @@
       </c>
       <c r="AQ5" s="19" cm="1">
         <f t="array" ref="AQ5">_xlfn.LET(_xlpm.r, AQ7:AQ90,SUM( _xlfn._xlws.FILTER( _xlpm.r, MOD(ROW(_xlpm.r) - ROW(INDEX(_xlpm.r,1,1)) + 1, 2) = 1 ) ))</f>
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="AR5" s="19" cm="1">
         <f t="array" ref="AR5">_xlfn.LET(_xlpm.r, AR7:AR90,SUM( _xlfn._xlws.FILTER( _xlpm.r, MOD(ROW(_xlpm.r) - ROW(INDEX(_xlpm.r,1,1)) + 1, 2) = 1 ) ))</f>
@@ -2940,8 +2959,8 @@
       </c>
     </row>
     <row r="6" spans="1:54" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A6" s="21" t="b">
-        <v>0</v>
+      <c r="A6" s="21" t="s">
+        <v>67</v>
       </c>
       <c r="B6" s="22" t="s">
         <v>13</v>
@@ -3010,7 +3029,7 @@
     </row>
     <row r="7" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="97" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B7" s="99" t="s">
         <v>31</v>
@@ -3085,7 +3104,7 @@
       <c r="C8" s="102"/>
       <c r="D8" s="104"/>
       <c r="E8" s="106"/>
-      <c r="F8" s="27">
+      <c r="F8" s="284">
         <v>1</v>
       </c>
       <c r="G8" s="28"/>
@@ -3138,21 +3157,21 @@
       <c r="BB8" s="29"/>
     </row>
     <row r="9" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="110" t="b">
-        <v>0</v>
-      </c>
-      <c r="B9" s="111" t="s">
+      <c r="A9" s="109" t="b">
+        <v>1</v>
+      </c>
+      <c r="B9" s="110" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="112">
+      <c r="C9" s="111">
         <f>SUM(F9:BB9)</f>
         <v>0.5</v>
       </c>
-      <c r="D9" s="112">
+      <c r="D9" s="111">
         <f>SUM(F10:BB10)</f>
         <v>0.5</v>
       </c>
-      <c r="E9" s="113">
+      <c r="E9" s="112">
         <f>(AVERAGE(C9,C10)-AVERAGE(D9,D10) )</f>
         <v>0</v>
       </c>
@@ -3215,7 +3234,7 @@
       <c r="D10" s="102"/>
       <c r="E10" s="106"/>
       <c r="F10" s="28"/>
-      <c r="G10" s="28">
+      <c r="G10" s="285">
         <v>0.5</v>
       </c>
       <c r="H10" s="28"/>
@@ -3267,21 +3286,21 @@
       <c r="BB10" s="29"/>
     </row>
     <row r="11" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A11" s="110" t="b">
-        <v>0</v>
-      </c>
-      <c r="B11" s="111" t="s">
+      <c r="A11" s="109" t="b">
+        <v>1</v>
+      </c>
+      <c r="B11" s="110" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="112">
+      <c r="C11" s="111">
         <f>SUM(F11:BB11)</f>
         <v>0.5</v>
       </c>
-      <c r="D11" s="112">
+      <c r="D11" s="111">
         <f>SUM(F12:BB12)</f>
         <v>0.5</v>
       </c>
-      <c r="E11" s="113">
+      <c r="E11" s="112">
         <f>(AVERAGE(C11,C12)-AVERAGE(D11,D12) )</f>
         <v>0</v>
       </c>
@@ -3344,7 +3363,7 @@
       <c r="D12" s="102"/>
       <c r="E12" s="106"/>
       <c r="F12" s="28"/>
-      <c r="G12" s="28">
+      <c r="G12" s="285">
         <v>0.5</v>
       </c>
       <c r="H12" s="28"/>
@@ -3396,21 +3415,21 @@
       <c r="BB12" s="29"/>
     </row>
     <row r="13" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="110" t="b">
-        <v>0</v>
-      </c>
-      <c r="B13" s="111" t="s">
+      <c r="A13" s="109" t="b">
+        <v>1</v>
+      </c>
+      <c r="B13" s="110" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="112">
+      <c r="C13" s="111">
         <f>SUM(F13:BB13)</f>
         <v>2.5</v>
       </c>
-      <c r="D13" s="112">
+      <c r="D13" s="111">
         <f>SUM(F14:BB14)</f>
         <v>2.5</v>
       </c>
-      <c r="E13" s="113">
+      <c r="E13" s="112">
         <f>(AVERAGE(C13,C14)-AVERAGE(D13,D14) )</f>
         <v>0</v>
       </c>
@@ -3477,13 +3496,13 @@
       <c r="D14" s="102"/>
       <c r="E14" s="106"/>
       <c r="F14" s="27"/>
-      <c r="G14" s="28">
+      <c r="G14" s="285">
         <v>0.5</v>
       </c>
-      <c r="H14" s="28">
+      <c r="H14" s="285">
         <v>1.5</v>
       </c>
-      <c r="I14" s="28">
+      <c r="I14" s="285">
         <v>0.5</v>
       </c>
       <c r="J14" s="29"/>
@@ -3533,142 +3552,142 @@
       <c r="BB14" s="29"/>
     </row>
     <row r="15" spans="1:54" x14ac:dyDescent="0.55000000000000004">
-      <c r="A15" s="124" t="b">
-        <v>0</v>
-      </c>
-      <c r="B15" s="126" t="s">
+      <c r="A15" s="123" t="b">
+        <v>1</v>
+      </c>
+      <c r="B15" s="125" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="128">
+      <c r="C15" s="127">
         <f>SUM(C17:C20)</f>
         <v>1</v>
       </c>
-      <c r="D15" s="128">
+      <c r="D15" s="127">
         <f>SUM(D17:D20)</f>
         <v>1</v>
       </c>
-      <c r="E15" s="130">
+      <c r="E15" s="129">
         <f>(C15-D15)</f>
         <v>0</v>
       </c>
-      <c r="F15" s="114"/>
-      <c r="G15" s="115"/>
-      <c r="H15" s="115"/>
-      <c r="I15" s="115"/>
-      <c r="J15" s="115"/>
-      <c r="K15" s="115"/>
-      <c r="L15" s="115"/>
-      <c r="M15" s="115"/>
-      <c r="N15" s="115"/>
-      <c r="O15" s="115"/>
-      <c r="P15" s="115"/>
-      <c r="Q15" s="115"/>
-      <c r="R15" s="115"/>
-      <c r="S15" s="115"/>
-      <c r="T15" s="115"/>
-      <c r="U15" s="115"/>
-      <c r="V15" s="115"/>
-      <c r="W15" s="115"/>
-      <c r="X15" s="115"/>
-      <c r="Y15" s="115"/>
-      <c r="Z15" s="115"/>
-      <c r="AA15" s="115"/>
-      <c r="AB15" s="115"/>
-      <c r="AC15" s="115"/>
-      <c r="AD15" s="115"/>
-      <c r="AE15" s="115"/>
-      <c r="AF15" s="115"/>
-      <c r="AG15" s="115"/>
-      <c r="AH15" s="115"/>
-      <c r="AI15" s="115"/>
-      <c r="AJ15" s="115"/>
-      <c r="AK15" s="115"/>
-      <c r="AL15" s="115"/>
-      <c r="AM15" s="115"/>
-      <c r="AN15" s="115"/>
-      <c r="AO15" s="115"/>
-      <c r="AP15" s="115"/>
-      <c r="AQ15" s="115"/>
-      <c r="AR15" s="115"/>
-      <c r="AS15" s="115"/>
-      <c r="AT15" s="115"/>
-      <c r="AU15" s="115"/>
-      <c r="AV15" s="115"/>
-      <c r="AW15" s="115"/>
-      <c r="AX15" s="115"/>
-      <c r="AY15" s="115"/>
-      <c r="AZ15" s="115"/>
-      <c r="BA15" s="115"/>
-      <c r="BB15" s="116"/>
+      <c r="F15" s="113"/>
+      <c r="G15" s="114"/>
+      <c r="H15" s="114"/>
+      <c r="I15" s="114"/>
+      <c r="J15" s="114"/>
+      <c r="K15" s="114"/>
+      <c r="L15" s="114"/>
+      <c r="M15" s="114"/>
+      <c r="N15" s="114"/>
+      <c r="O15" s="114"/>
+      <c r="P15" s="114"/>
+      <c r="Q15" s="114"/>
+      <c r="R15" s="114"/>
+      <c r="S15" s="114"/>
+      <c r="T15" s="114"/>
+      <c r="U15" s="114"/>
+      <c r="V15" s="114"/>
+      <c r="W15" s="114"/>
+      <c r="X15" s="114"/>
+      <c r="Y15" s="114"/>
+      <c r="Z15" s="114"/>
+      <c r="AA15" s="114"/>
+      <c r="AB15" s="114"/>
+      <c r="AC15" s="114"/>
+      <c r="AD15" s="114"/>
+      <c r="AE15" s="114"/>
+      <c r="AF15" s="114"/>
+      <c r="AG15" s="114"/>
+      <c r="AH15" s="114"/>
+      <c r="AI15" s="114"/>
+      <c r="AJ15" s="114"/>
+      <c r="AK15" s="114"/>
+      <c r="AL15" s="114"/>
+      <c r="AM15" s="114"/>
+      <c r="AN15" s="114"/>
+      <c r="AO15" s="114"/>
+      <c r="AP15" s="114"/>
+      <c r="AQ15" s="114"/>
+      <c r="AR15" s="114"/>
+      <c r="AS15" s="114"/>
+      <c r="AT15" s="114"/>
+      <c r="AU15" s="114"/>
+      <c r="AV15" s="114"/>
+      <c r="AW15" s="114"/>
+      <c r="AX15" s="114"/>
+      <c r="AY15" s="114"/>
+      <c r="AZ15" s="114"/>
+      <c r="BA15" s="114"/>
+      <c r="BB15" s="115"/>
     </row>
     <row r="16" spans="1:54" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A16" s="125"/>
-      <c r="B16" s="127"/>
-      <c r="C16" s="129"/>
-      <c r="D16" s="129"/>
-      <c r="E16" s="131"/>
-      <c r="F16" s="117"/>
-      <c r="G16" s="118"/>
-      <c r="H16" s="118"/>
-      <c r="I16" s="118"/>
-      <c r="J16" s="118"/>
-      <c r="K16" s="118"/>
-      <c r="L16" s="118"/>
-      <c r="M16" s="118"/>
-      <c r="N16" s="118"/>
-      <c r="O16" s="118"/>
-      <c r="P16" s="118"/>
-      <c r="Q16" s="118"/>
-      <c r="R16" s="118"/>
-      <c r="S16" s="118"/>
-      <c r="T16" s="118"/>
-      <c r="U16" s="118"/>
-      <c r="V16" s="118"/>
-      <c r="W16" s="118"/>
-      <c r="X16" s="118"/>
-      <c r="Y16" s="118"/>
-      <c r="Z16" s="118"/>
-      <c r="AA16" s="118"/>
-      <c r="AB16" s="118"/>
-      <c r="AC16" s="118"/>
-      <c r="AD16" s="118"/>
-      <c r="AE16" s="118"/>
-      <c r="AF16" s="118"/>
-      <c r="AG16" s="118"/>
-      <c r="AH16" s="118"/>
-      <c r="AI16" s="118"/>
-      <c r="AJ16" s="118"/>
-      <c r="AK16" s="118"/>
-      <c r="AL16" s="118"/>
-      <c r="AM16" s="118"/>
-      <c r="AN16" s="118"/>
-      <c r="AO16" s="118"/>
-      <c r="AP16" s="118"/>
-      <c r="AQ16" s="118"/>
-      <c r="AR16" s="118"/>
-      <c r="AS16" s="118"/>
-      <c r="AT16" s="118"/>
-      <c r="AU16" s="118"/>
-      <c r="AV16" s="118"/>
-      <c r="AW16" s="118"/>
-      <c r="AX16" s="118"/>
-      <c r="AY16" s="118"/>
-      <c r="AZ16" s="118"/>
-      <c r="BA16" s="118"/>
-      <c r="BB16" s="119"/>
+      <c r="A16" s="124"/>
+      <c r="B16" s="126"/>
+      <c r="C16" s="128"/>
+      <c r="D16" s="128"/>
+      <c r="E16" s="130"/>
+      <c r="F16" s="116"/>
+      <c r="G16" s="117"/>
+      <c r="H16" s="117"/>
+      <c r="I16" s="117"/>
+      <c r="J16" s="117"/>
+      <c r="K16" s="117"/>
+      <c r="L16" s="117"/>
+      <c r="M16" s="117"/>
+      <c r="N16" s="117"/>
+      <c r="O16" s="117"/>
+      <c r="P16" s="117"/>
+      <c r="Q16" s="117"/>
+      <c r="R16" s="117"/>
+      <c r="S16" s="117"/>
+      <c r="T16" s="117"/>
+      <c r="U16" s="117"/>
+      <c r="V16" s="117"/>
+      <c r="W16" s="117"/>
+      <c r="X16" s="117"/>
+      <c r="Y16" s="117"/>
+      <c r="Z16" s="117"/>
+      <c r="AA16" s="117"/>
+      <c r="AB16" s="117"/>
+      <c r="AC16" s="117"/>
+      <c r="AD16" s="117"/>
+      <c r="AE16" s="117"/>
+      <c r="AF16" s="117"/>
+      <c r="AG16" s="117"/>
+      <c r="AH16" s="117"/>
+      <c r="AI16" s="117"/>
+      <c r="AJ16" s="117"/>
+      <c r="AK16" s="117"/>
+      <c r="AL16" s="117"/>
+      <c r="AM16" s="117"/>
+      <c r="AN16" s="117"/>
+      <c r="AO16" s="117"/>
+      <c r="AP16" s="117"/>
+      <c r="AQ16" s="117"/>
+      <c r="AR16" s="117"/>
+      <c r="AS16" s="117"/>
+      <c r="AT16" s="117"/>
+      <c r="AU16" s="117"/>
+      <c r="AV16" s="117"/>
+      <c r="AW16" s="117"/>
+      <c r="AX16" s="117"/>
+      <c r="AY16" s="117"/>
+      <c r="AZ16" s="117"/>
+      <c r="BA16" s="117"/>
+      <c r="BB16" s="118"/>
     </row>
     <row r="17" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A17" s="120" t="b">
-        <v>0</v>
-      </c>
-      <c r="B17" s="122" t="s">
-        <v>55</v>
-      </c>
-      <c r="C17" s="112">
+      <c r="A17" s="119" t="b">
+        <v>1</v>
+      </c>
+      <c r="B17" s="121" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" s="111">
         <f>SUM(F17:BB17)</f>
         <v>0.5</v>
       </c>
-      <c r="D17" s="112">
+      <c r="D17" s="111">
         <f>SUM(F18:BB18)</f>
         <v>0.5</v>
       </c>
@@ -3729,15 +3748,15 @@
       <c r="BB17" s="26"/>
     </row>
     <row r="18" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A18" s="121"/>
-      <c r="B18" s="123"/>
+      <c r="A18" s="120"/>
+      <c r="B18" s="122"/>
       <c r="C18" s="102"/>
       <c r="D18" s="102"/>
       <c r="E18" s="106"/>
       <c r="F18" s="27"/>
       <c r="G18" s="28"/>
       <c r="H18" s="28"/>
-      <c r="I18" s="28">
+      <c r="I18" s="285">
         <v>0.5</v>
       </c>
       <c r="J18" s="29"/>
@@ -3787,21 +3806,21 @@
       <c r="BB18" s="29"/>
     </row>
     <row r="19" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="142" t="b">
-        <v>0</v>
-      </c>
-      <c r="B19" s="143" t="s">
-        <v>54</v>
-      </c>
-      <c r="C19" s="112">
+      <c r="A19" s="141" t="b">
+        <v>1</v>
+      </c>
+      <c r="B19" s="287" t="s">
+        <v>66</v>
+      </c>
+      <c r="C19" s="111">
         <f>SUM(F19:BB19)</f>
         <v>0.5</v>
       </c>
-      <c r="D19" s="112">
+      <c r="D19" s="111">
         <f>SUM(F20:BB20)</f>
         <v>0.5</v>
       </c>
-      <c r="E19" s="113">
+      <c r="E19" s="112">
         <f>(AVERAGE(C19,C20)-AVERAGE(D19,D20) )</f>
         <v>0</v>
       </c>
@@ -3858,15 +3877,15 @@
       <c r="BB19" s="32"/>
     </row>
     <row r="20" spans="1:54" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A20" s="121"/>
-      <c r="B20" s="144"/>
+      <c r="A20" s="120"/>
+      <c r="B20" s="142"/>
       <c r="C20" s="102"/>
       <c r="D20" s="102"/>
-      <c r="E20" s="145"/>
+      <c r="E20" s="143"/>
       <c r="F20" s="25"/>
       <c r="G20" s="58"/>
       <c r="H20" s="58"/>
-      <c r="I20" s="58">
+      <c r="I20" s="286">
         <v>0.5</v>
       </c>
       <c r="J20" s="26"/>
@@ -3916,155 +3935,155 @@
       <c r="BB20" s="26"/>
     </row>
     <row r="21" spans="1:54" ht="18" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A21" s="146" t="b">
-        <v>0</v>
-      </c>
-      <c r="B21" s="148" t="s">
+      <c r="A21" s="144" t="b">
+        <v>0</v>
+      </c>
+      <c r="B21" s="146" t="s">
         <v>15</v>
       </c>
-      <c r="C21" s="150">
+      <c r="C21" s="148">
         <f>SUM(C23:C28)</f>
         <v>3</v>
       </c>
-      <c r="D21" s="150">
+      <c r="D21" s="148">
         <f>SUM(D23:D28)</f>
-        <v>0</v>
-      </c>
-      <c r="E21" s="152">
+        <v>2.5</v>
+      </c>
+      <c r="E21" s="150">
         <f>(C21-D21)</f>
-        <v>3</v>
-      </c>
-      <c r="F21" s="132"/>
-      <c r="G21" s="133"/>
-      <c r="H21" s="133"/>
-      <c r="I21" s="133"/>
-      <c r="J21" s="133"/>
-      <c r="K21" s="133"/>
-      <c r="L21" s="133"/>
-      <c r="M21" s="133"/>
-      <c r="N21" s="133"/>
-      <c r="O21" s="133"/>
-      <c r="P21" s="133"/>
-      <c r="Q21" s="133"/>
-      <c r="R21" s="133"/>
-      <c r="S21" s="133"/>
-      <c r="T21" s="133"/>
-      <c r="U21" s="133"/>
-      <c r="V21" s="133"/>
-      <c r="W21" s="133"/>
-      <c r="X21" s="133"/>
-      <c r="Y21" s="133"/>
-      <c r="Z21" s="133"/>
-      <c r="AA21" s="133"/>
-      <c r="AB21" s="133"/>
-      <c r="AC21" s="133"/>
-      <c r="AD21" s="133"/>
-      <c r="AE21" s="133"/>
-      <c r="AF21" s="133"/>
-      <c r="AG21" s="133"/>
-      <c r="AH21" s="133"/>
-      <c r="AI21" s="133"/>
-      <c r="AJ21" s="133"/>
-      <c r="AK21" s="133"/>
-      <c r="AL21" s="133"/>
-      <c r="AM21" s="133"/>
-      <c r="AN21" s="133"/>
-      <c r="AO21" s="133"/>
-      <c r="AP21" s="133"/>
-      <c r="AQ21" s="133"/>
-      <c r="AR21" s="133"/>
-      <c r="AS21" s="133"/>
-      <c r="AT21" s="133"/>
-      <c r="AU21" s="133"/>
-      <c r="AV21" s="133"/>
-      <c r="AW21" s="133"/>
-      <c r="AX21" s="133"/>
-      <c r="AY21" s="133"/>
-      <c r="AZ21" s="133"/>
-      <c r="BA21" s="133"/>
-      <c r="BB21" s="134"/>
+        <v>0.5</v>
+      </c>
+      <c r="F21" s="131"/>
+      <c r="G21" s="132"/>
+      <c r="H21" s="132"/>
+      <c r="I21" s="132"/>
+      <c r="J21" s="132"/>
+      <c r="K21" s="132"/>
+      <c r="L21" s="132"/>
+      <c r="M21" s="132"/>
+      <c r="N21" s="132"/>
+      <c r="O21" s="132"/>
+      <c r="P21" s="132"/>
+      <c r="Q21" s="132"/>
+      <c r="R21" s="132"/>
+      <c r="S21" s="132"/>
+      <c r="T21" s="132"/>
+      <c r="U21" s="132"/>
+      <c r="V21" s="132"/>
+      <c r="W21" s="132"/>
+      <c r="X21" s="132"/>
+      <c r="Y21" s="132"/>
+      <c r="Z21" s="132"/>
+      <c r="AA21" s="132"/>
+      <c r="AB21" s="132"/>
+      <c r="AC21" s="132"/>
+      <c r="AD21" s="132"/>
+      <c r="AE21" s="132"/>
+      <c r="AF21" s="132"/>
+      <c r="AG21" s="132"/>
+      <c r="AH21" s="132"/>
+      <c r="AI21" s="132"/>
+      <c r="AJ21" s="132"/>
+      <c r="AK21" s="132"/>
+      <c r="AL21" s="132"/>
+      <c r="AM21" s="132"/>
+      <c r="AN21" s="132"/>
+      <c r="AO21" s="132"/>
+      <c r="AP21" s="132"/>
+      <c r="AQ21" s="132"/>
+      <c r="AR21" s="132"/>
+      <c r="AS21" s="132"/>
+      <c r="AT21" s="132"/>
+      <c r="AU21" s="132"/>
+      <c r="AV21" s="132"/>
+      <c r="AW21" s="132"/>
+      <c r="AX21" s="132"/>
+      <c r="AY21" s="132"/>
+      <c r="AZ21" s="132"/>
+      <c r="BA21" s="132"/>
+      <c r="BB21" s="133"/>
     </row>
     <row r="22" spans="1:54" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A22" s="147"/>
-      <c r="B22" s="149"/>
-      <c r="C22" s="151"/>
-      <c r="D22" s="151"/>
-      <c r="E22" s="153"/>
-      <c r="F22" s="135"/>
-      <c r="G22" s="136"/>
-      <c r="H22" s="136"/>
-      <c r="I22" s="136"/>
-      <c r="J22" s="136"/>
-      <c r="K22" s="136"/>
-      <c r="L22" s="136"/>
-      <c r="M22" s="136"/>
-      <c r="N22" s="136"/>
-      <c r="O22" s="136"/>
-      <c r="P22" s="136"/>
-      <c r="Q22" s="136"/>
-      <c r="R22" s="136"/>
-      <c r="S22" s="136"/>
-      <c r="T22" s="136"/>
-      <c r="U22" s="136"/>
-      <c r="V22" s="136"/>
-      <c r="W22" s="136"/>
-      <c r="X22" s="136"/>
-      <c r="Y22" s="136"/>
-      <c r="Z22" s="136"/>
-      <c r="AA22" s="136"/>
-      <c r="AB22" s="136"/>
-      <c r="AC22" s="136"/>
-      <c r="AD22" s="136"/>
-      <c r="AE22" s="136"/>
-      <c r="AF22" s="136"/>
-      <c r="AG22" s="136"/>
-      <c r="AH22" s="136"/>
-      <c r="AI22" s="136"/>
-      <c r="AJ22" s="136"/>
-      <c r="AK22" s="136"/>
-      <c r="AL22" s="136"/>
-      <c r="AM22" s="136"/>
-      <c r="AN22" s="136"/>
-      <c r="AO22" s="136"/>
-      <c r="AP22" s="136"/>
-      <c r="AQ22" s="136"/>
-      <c r="AR22" s="136"/>
-      <c r="AS22" s="136"/>
-      <c r="AT22" s="136"/>
-      <c r="AU22" s="136"/>
-      <c r="AV22" s="136"/>
-      <c r="AW22" s="136"/>
-      <c r="AX22" s="136"/>
-      <c r="AY22" s="136"/>
-      <c r="AZ22" s="136"/>
-      <c r="BA22" s="136"/>
-      <c r="BB22" s="137"/>
+      <c r="A22" s="145"/>
+      <c r="B22" s="147"/>
+      <c r="C22" s="149"/>
+      <c r="D22" s="149"/>
+      <c r="E22" s="151"/>
+      <c r="F22" s="134"/>
+      <c r="G22" s="135"/>
+      <c r="H22" s="135"/>
+      <c r="I22" s="135"/>
+      <c r="J22" s="135"/>
+      <c r="K22" s="135"/>
+      <c r="L22" s="135"/>
+      <c r="M22" s="135"/>
+      <c r="N22" s="135"/>
+      <c r="O22" s="135"/>
+      <c r="P22" s="135"/>
+      <c r="Q22" s="135"/>
+      <c r="R22" s="135"/>
+      <c r="S22" s="135"/>
+      <c r="T22" s="135"/>
+      <c r="U22" s="135"/>
+      <c r="V22" s="135"/>
+      <c r="W22" s="135"/>
+      <c r="X22" s="135"/>
+      <c r="Y22" s="135"/>
+      <c r="Z22" s="135"/>
+      <c r="AA22" s="135"/>
+      <c r="AB22" s="135"/>
+      <c r="AC22" s="135"/>
+      <c r="AD22" s="135"/>
+      <c r="AE22" s="135"/>
+      <c r="AF22" s="135"/>
+      <c r="AG22" s="135"/>
+      <c r="AH22" s="135"/>
+      <c r="AI22" s="135"/>
+      <c r="AJ22" s="135"/>
+      <c r="AK22" s="135"/>
+      <c r="AL22" s="135"/>
+      <c r="AM22" s="135"/>
+      <c r="AN22" s="135"/>
+      <c r="AO22" s="135"/>
+      <c r="AP22" s="135"/>
+      <c r="AQ22" s="135"/>
+      <c r="AR22" s="135"/>
+      <c r="AS22" s="135"/>
+      <c r="AT22" s="135"/>
+      <c r="AU22" s="135"/>
+      <c r="AV22" s="135"/>
+      <c r="AW22" s="135"/>
+      <c r="AX22" s="135"/>
+      <c r="AY22" s="135"/>
+      <c r="AZ22" s="135"/>
+      <c r="BA22" s="135"/>
+      <c r="BB22" s="136"/>
     </row>
     <row r="23" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A23" s="138" t="b">
-        <v>0</v>
-      </c>
-      <c r="B23" s="140" t="s">
+      <c r="A23" s="137" t="b">
+        <v>1</v>
+      </c>
+      <c r="B23" s="139" t="s">
         <v>33</v>
       </c>
-      <c r="C23" s="112">
+      <c r="C23" s="111">
         <f>SUM(F23:BB23)</f>
         <v>1</v>
       </c>
-      <c r="D23" s="112">
+      <c r="D23" s="111">
         <f>SUM(F24:BB24)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E23" s="105">
         <f>(AVERAGE(C23,C24)-AVERAGE(D23,D24) )</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F23" s="33"/>
       <c r="G23" s="62"/>
       <c r="H23" s="62"/>
       <c r="I23" s="62"/>
       <c r="J23" s="34" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K23" s="64">
         <v>1</v>
@@ -4114,8 +4133,8 @@
       <c r="BB23" s="26"/>
     </row>
     <row r="24" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A24" s="139"/>
-      <c r="B24" s="141"/>
+      <c r="A24" s="138"/>
+      <c r="B24" s="140"/>
       <c r="C24" s="102"/>
       <c r="D24" s="102"/>
       <c r="E24" s="106"/>
@@ -4124,7 +4143,9 @@
       <c r="H24" s="36"/>
       <c r="I24" s="36"/>
       <c r="J24" s="37"/>
-      <c r="K24" s="27"/>
+      <c r="K24" s="27">
+        <v>1</v>
+      </c>
       <c r="L24" s="28"/>
       <c r="M24" s="28"/>
       <c r="N24" s="28"/>
@@ -4170,23 +4191,23 @@
       <c r="BB24" s="29"/>
     </row>
     <row r="25" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A25" s="168" t="b">
-        <v>0</v>
-      </c>
-      <c r="B25" s="169" t="s">
+      <c r="A25" s="166" t="b">
+        <v>0</v>
+      </c>
+      <c r="B25" s="167" t="s">
         <v>34</v>
       </c>
-      <c r="C25" s="112">
+      <c r="C25" s="111">
         <f>SUM(F25:BB25)</f>
         <v>1</v>
       </c>
-      <c r="D25" s="112">
+      <c r="D25" s="111">
         <f>SUM(F26:BB26)</f>
-        <v>0</v>
-      </c>
-      <c r="E25" s="113">
+        <v>0.5</v>
+      </c>
+      <c r="E25" s="112">
         <f>(AVERAGE(C25,C26)-AVERAGE(D25,D26) )</f>
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F25" s="33"/>
       <c r="G25" s="62"/>
@@ -4241,8 +4262,8 @@
       <c r="BB25" s="26"/>
     </row>
     <row r="26" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="139"/>
-      <c r="B26" s="141"/>
+      <c r="A26" s="138"/>
+      <c r="B26" s="140"/>
       <c r="C26" s="102"/>
       <c r="D26" s="102"/>
       <c r="E26" s="106"/>
@@ -4251,8 +4272,12 @@
       <c r="H26" s="36"/>
       <c r="I26" s="36"/>
       <c r="J26" s="37"/>
-      <c r="K26" s="27"/>
-      <c r="L26" s="28"/>
+      <c r="K26" s="27">
+        <v>0.3</v>
+      </c>
+      <c r="L26" s="28">
+        <v>0.2</v>
+      </c>
       <c r="M26" s="28"/>
       <c r="N26" s="28"/>
       <c r="O26" s="29"/>
@@ -4297,23 +4322,23 @@
       <c r="BB26" s="29"/>
     </row>
     <row r="27" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A27" s="168" t="b">
-        <v>0</v>
-      </c>
-      <c r="B27" s="169" t="s">
+      <c r="A27" s="166" t="b">
+        <v>0</v>
+      </c>
+      <c r="B27" s="167" t="s">
         <v>35</v>
       </c>
-      <c r="C27" s="112">
+      <c r="C27" s="111">
         <f>SUM(F27:BB27)</f>
         <v>1</v>
       </c>
-      <c r="D27" s="112">
+      <c r="D27" s="111">
         <f>SUM(F28:BB28)</f>
-        <v>0</v>
-      </c>
-      <c r="E27" s="113">
+        <v>1</v>
+      </c>
+      <c r="E27" s="112">
         <f>(AVERAGE(C27,C28)-AVERAGE(D27,D28) )</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F27" s="33"/>
       <c r="G27" s="62"/>
@@ -4368,18 +4393,20 @@
       <c r="BB27" s="32"/>
     </row>
     <row r="28" spans="1:54" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A28" s="139"/>
-      <c r="B28" s="141"/>
+      <c r="A28" s="138"/>
+      <c r="B28" s="140"/>
       <c r="C28" s="102"/>
       <c r="D28" s="102"/>
-      <c r="E28" s="145"/>
+      <c r="E28" s="143"/>
       <c r="F28" s="33"/>
       <c r="G28" s="62"/>
       <c r="H28" s="62"/>
       <c r="I28" s="62"/>
       <c r="J28" s="34"/>
       <c r="K28" s="25"/>
-      <c r="L28" s="58"/>
+      <c r="L28" s="58">
+        <v>1</v>
+      </c>
       <c r="M28" s="58"/>
       <c r="N28" s="58"/>
       <c r="O28" s="26"/>
@@ -4424,142 +4451,142 @@
       <c r="BB28" s="26"/>
     </row>
     <row r="29" spans="1:54" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A29" s="154" t="b">
-        <v>0</v>
-      </c>
-      <c r="B29" s="156" t="s">
+      <c r="A29" s="152" t="b">
+        <v>0</v>
+      </c>
+      <c r="B29" s="154" t="s">
         <v>16</v>
       </c>
-      <c r="C29" s="158">
+      <c r="C29" s="156">
         <f>SUM(C31:C40)</f>
         <v>7.5</v>
       </c>
-      <c r="D29" s="158">
+      <c r="D29" s="156">
         <f>SUM(D31:D40)</f>
         <v>0</v>
       </c>
-      <c r="E29" s="160">
+      <c r="E29" s="158">
         <f>(C29-D29)</f>
         <v>7.5</v>
       </c>
-      <c r="F29" s="162"/>
-      <c r="G29" s="163"/>
-      <c r="H29" s="163"/>
-      <c r="I29" s="163"/>
-      <c r="J29" s="163"/>
-      <c r="K29" s="163"/>
-      <c r="L29" s="163"/>
-      <c r="M29" s="163"/>
-      <c r="N29" s="163"/>
-      <c r="O29" s="163"/>
-      <c r="P29" s="163"/>
-      <c r="Q29" s="163"/>
-      <c r="R29" s="163"/>
-      <c r="S29" s="163"/>
-      <c r="T29" s="163"/>
-      <c r="U29" s="163"/>
-      <c r="V29" s="163"/>
-      <c r="W29" s="163"/>
-      <c r="X29" s="163"/>
-      <c r="Y29" s="163"/>
-      <c r="Z29" s="163"/>
-      <c r="AA29" s="163"/>
-      <c r="AB29" s="163"/>
-      <c r="AC29" s="163"/>
-      <c r="AD29" s="163"/>
-      <c r="AE29" s="163"/>
-      <c r="AF29" s="163"/>
-      <c r="AG29" s="163"/>
-      <c r="AH29" s="163"/>
-      <c r="AI29" s="163"/>
-      <c r="AJ29" s="163"/>
-      <c r="AK29" s="163"/>
-      <c r="AL29" s="163"/>
-      <c r="AM29" s="163"/>
-      <c r="AN29" s="163"/>
-      <c r="AO29" s="163"/>
-      <c r="AP29" s="163"/>
-      <c r="AQ29" s="163"/>
-      <c r="AR29" s="163"/>
-      <c r="AS29" s="163"/>
-      <c r="AT29" s="163"/>
-      <c r="AU29" s="163"/>
-      <c r="AV29" s="163"/>
-      <c r="AW29" s="163"/>
-      <c r="AX29" s="163"/>
-      <c r="AY29" s="163"/>
-      <c r="AZ29" s="163"/>
-      <c r="BA29" s="163"/>
-      <c r="BB29" s="164"/>
+      <c r="F29" s="160"/>
+      <c r="G29" s="161"/>
+      <c r="H29" s="161"/>
+      <c r="I29" s="161"/>
+      <c r="J29" s="161"/>
+      <c r="K29" s="161"/>
+      <c r="L29" s="161"/>
+      <c r="M29" s="161"/>
+      <c r="N29" s="161"/>
+      <c r="O29" s="161"/>
+      <c r="P29" s="161"/>
+      <c r="Q29" s="161"/>
+      <c r="R29" s="161"/>
+      <c r="S29" s="161"/>
+      <c r="T29" s="161"/>
+      <c r="U29" s="161"/>
+      <c r="V29" s="161"/>
+      <c r="W29" s="161"/>
+      <c r="X29" s="161"/>
+      <c r="Y29" s="161"/>
+      <c r="Z29" s="161"/>
+      <c r="AA29" s="161"/>
+      <c r="AB29" s="161"/>
+      <c r="AC29" s="161"/>
+      <c r="AD29" s="161"/>
+      <c r="AE29" s="161"/>
+      <c r="AF29" s="161"/>
+      <c r="AG29" s="161"/>
+      <c r="AH29" s="161"/>
+      <c r="AI29" s="161"/>
+      <c r="AJ29" s="161"/>
+      <c r="AK29" s="161"/>
+      <c r="AL29" s="161"/>
+      <c r="AM29" s="161"/>
+      <c r="AN29" s="161"/>
+      <c r="AO29" s="161"/>
+      <c r="AP29" s="161"/>
+      <c r="AQ29" s="161"/>
+      <c r="AR29" s="161"/>
+      <c r="AS29" s="161"/>
+      <c r="AT29" s="161"/>
+      <c r="AU29" s="161"/>
+      <c r="AV29" s="161"/>
+      <c r="AW29" s="161"/>
+      <c r="AX29" s="161"/>
+      <c r="AY29" s="161"/>
+      <c r="AZ29" s="161"/>
+      <c r="BA29" s="161"/>
+      <c r="BB29" s="162"/>
     </row>
     <row r="30" spans="1:54" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A30" s="155"/>
-      <c r="B30" s="157"/>
-      <c r="C30" s="159"/>
-      <c r="D30" s="159"/>
-      <c r="E30" s="161"/>
-      <c r="F30" s="165"/>
-      <c r="G30" s="166"/>
-      <c r="H30" s="166"/>
-      <c r="I30" s="166"/>
-      <c r="J30" s="166"/>
-      <c r="K30" s="166"/>
-      <c r="L30" s="166"/>
-      <c r="M30" s="166"/>
-      <c r="N30" s="166"/>
-      <c r="O30" s="166"/>
-      <c r="P30" s="166"/>
-      <c r="Q30" s="166"/>
-      <c r="R30" s="166"/>
-      <c r="S30" s="166"/>
-      <c r="T30" s="166"/>
-      <c r="U30" s="166"/>
-      <c r="V30" s="166"/>
-      <c r="W30" s="166"/>
-      <c r="X30" s="166"/>
-      <c r="Y30" s="166"/>
-      <c r="Z30" s="166"/>
-      <c r="AA30" s="166"/>
-      <c r="AB30" s="166"/>
-      <c r="AC30" s="166"/>
-      <c r="AD30" s="166"/>
-      <c r="AE30" s="166"/>
-      <c r="AF30" s="166"/>
-      <c r="AG30" s="166"/>
-      <c r="AH30" s="166"/>
-      <c r="AI30" s="166"/>
-      <c r="AJ30" s="166"/>
-      <c r="AK30" s="166"/>
-      <c r="AL30" s="166"/>
-      <c r="AM30" s="166"/>
-      <c r="AN30" s="166"/>
-      <c r="AO30" s="166"/>
-      <c r="AP30" s="166"/>
-      <c r="AQ30" s="166"/>
-      <c r="AR30" s="166"/>
-      <c r="AS30" s="166"/>
-      <c r="AT30" s="166"/>
-      <c r="AU30" s="166"/>
-      <c r="AV30" s="166"/>
-      <c r="AW30" s="166"/>
-      <c r="AX30" s="166"/>
-      <c r="AY30" s="166"/>
-      <c r="AZ30" s="166"/>
-      <c r="BA30" s="166"/>
-      <c r="BB30" s="167"/>
+      <c r="A30" s="153"/>
+      <c r="B30" s="155"/>
+      <c r="C30" s="157"/>
+      <c r="D30" s="157"/>
+      <c r="E30" s="159"/>
+      <c r="F30" s="163"/>
+      <c r="G30" s="164"/>
+      <c r="H30" s="164"/>
+      <c r="I30" s="164"/>
+      <c r="J30" s="164"/>
+      <c r="K30" s="164"/>
+      <c r="L30" s="164"/>
+      <c r="M30" s="164"/>
+      <c r="N30" s="164"/>
+      <c r="O30" s="164"/>
+      <c r="P30" s="164"/>
+      <c r="Q30" s="164"/>
+      <c r="R30" s="164"/>
+      <c r="S30" s="164"/>
+      <c r="T30" s="164"/>
+      <c r="U30" s="164"/>
+      <c r="V30" s="164"/>
+      <c r="W30" s="164"/>
+      <c r="X30" s="164"/>
+      <c r="Y30" s="164"/>
+      <c r="Z30" s="164"/>
+      <c r="AA30" s="164"/>
+      <c r="AB30" s="164"/>
+      <c r="AC30" s="164"/>
+      <c r="AD30" s="164"/>
+      <c r="AE30" s="164"/>
+      <c r="AF30" s="164"/>
+      <c r="AG30" s="164"/>
+      <c r="AH30" s="164"/>
+      <c r="AI30" s="164"/>
+      <c r="AJ30" s="164"/>
+      <c r="AK30" s="164"/>
+      <c r="AL30" s="164"/>
+      <c r="AM30" s="164"/>
+      <c r="AN30" s="164"/>
+      <c r="AO30" s="164"/>
+      <c r="AP30" s="164"/>
+      <c r="AQ30" s="164"/>
+      <c r="AR30" s="164"/>
+      <c r="AS30" s="164"/>
+      <c r="AT30" s="164"/>
+      <c r="AU30" s="164"/>
+      <c r="AV30" s="164"/>
+      <c r="AW30" s="164"/>
+      <c r="AX30" s="164"/>
+      <c r="AY30" s="164"/>
+      <c r="AZ30" s="164"/>
+      <c r="BA30" s="164"/>
+      <c r="BB30" s="165"/>
     </row>
     <row r="31" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="170" t="b">
-        <v>0</v>
-      </c>
-      <c r="B31" s="172" t="s">
+      <c r="A31" s="168" t="b">
+        <v>0</v>
+      </c>
+      <c r="B31" s="170" t="s">
         <v>39</v>
       </c>
-      <c r="C31" s="112">
+      <c r="C31" s="111">
         <f>SUM(F31:BB31)</f>
         <v>1.5</v>
       </c>
-      <c r="D31" s="112">
+      <c r="D31" s="111">
         <f>SUM(F32:BB32)</f>
         <v>0</v>
       </c>
@@ -4624,8 +4651,8 @@
       <c r="BB31" s="26"/>
     </row>
     <row r="32" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="171"/>
-      <c r="B32" s="173"/>
+      <c r="A32" s="169"/>
+      <c r="B32" s="171"/>
       <c r="C32" s="102"/>
       <c r="D32" s="102"/>
       <c r="E32" s="106"/>
@@ -4680,21 +4707,21 @@
       <c r="BB32" s="29"/>
     </row>
     <row r="33" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" s="174" t="b">
-        <v>0</v>
-      </c>
-      <c r="B33" s="175" t="s">
+      <c r="A33" s="172" t="b">
+        <v>0</v>
+      </c>
+      <c r="B33" s="173" t="s">
         <v>40</v>
       </c>
-      <c r="C33" s="112">
+      <c r="C33" s="111">
         <f>SUM(F33:BB33)</f>
         <v>1</v>
       </c>
-      <c r="D33" s="112">
+      <c r="D33" s="111">
         <f>SUM(F34:BB34)</f>
         <v>0</v>
       </c>
-      <c r="E33" s="113">
+      <c r="E33" s="112">
         <f>(AVERAGE(C33,C34)-AVERAGE(D33,D34) )</f>
         <v>1</v>
       </c>
@@ -4751,8 +4778,8 @@
       <c r="BB33" s="32"/>
     </row>
     <row r="34" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="171"/>
-      <c r="B34" s="173"/>
+      <c r="A34" s="169"/>
+      <c r="B34" s="171"/>
       <c r="C34" s="102"/>
       <c r="D34" s="102"/>
       <c r="E34" s="106"/>
@@ -4807,21 +4834,21 @@
       <c r="BB34" s="29"/>
     </row>
     <row r="35" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A35" s="174" t="b">
-        <v>0</v>
-      </c>
-      <c r="B35" s="175" t="s">
+      <c r="A35" s="172" t="b">
+        <v>0</v>
+      </c>
+      <c r="B35" s="173" t="s">
         <v>36</v>
       </c>
-      <c r="C35" s="112">
+      <c r="C35" s="111">
         <f>SUM(F35:BB35)</f>
         <v>2</v>
       </c>
-      <c r="D35" s="112">
+      <c r="D35" s="111">
         <f>SUM(F36:BB36)</f>
         <v>0</v>
       </c>
-      <c r="E35" s="113">
+      <c r="E35" s="112">
         <f t="shared" ref="E35" si="0">(AVERAGE(C35,C36)-AVERAGE(D35,D36) )</f>
         <v>2</v>
       </c>
@@ -4878,8 +4905,8 @@
       <c r="BB35" s="32"/>
     </row>
     <row r="36" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A36" s="171"/>
-      <c r="B36" s="173"/>
+      <c r="A36" s="169"/>
+      <c r="B36" s="171"/>
       <c r="C36" s="102"/>
       <c r="D36" s="102"/>
       <c r="E36" s="106"/>
@@ -4934,21 +4961,21 @@
       <c r="BB36" s="29"/>
     </row>
     <row r="37" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A37" s="174" t="b">
-        <v>0</v>
-      </c>
-      <c r="B37" s="175" t="s">
+      <c r="A37" s="172" t="b">
+        <v>0</v>
+      </c>
+      <c r="B37" s="173" t="s">
         <v>41</v>
       </c>
-      <c r="C37" s="112">
+      <c r="C37" s="111">
         <f>SUM(F37:BB37)</f>
         <v>0.5</v>
       </c>
-      <c r="D37" s="112">
+      <c r="D37" s="111">
         <f>SUM(F38:BB38)</f>
         <v>0</v>
       </c>
-      <c r="E37" s="113">
+      <c r="E37" s="112">
         <f t="shared" ref="E37" si="1">(AVERAGE(C37,C38)-AVERAGE(D37,D38) )</f>
         <v>0.5</v>
       </c>
@@ -5005,8 +5032,8 @@
       <c r="BB37" s="32"/>
     </row>
     <row r="38" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A38" s="171"/>
-      <c r="B38" s="173"/>
+      <c r="A38" s="169"/>
+      <c r="B38" s="171"/>
       <c r="C38" s="102"/>
       <c r="D38" s="102"/>
       <c r="E38" s="106"/>
@@ -5061,21 +5088,21 @@
       <c r="BB38" s="29"/>
     </row>
     <row r="39" spans="1:54" ht="13.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A39" s="174" t="b">
-        <v>0</v>
-      </c>
-      <c r="B39" s="175" t="s">
+      <c r="A39" s="172" t="b">
+        <v>0</v>
+      </c>
+      <c r="B39" s="173" t="s">
         <v>53</v>
       </c>
-      <c r="C39" s="112">
+      <c r="C39" s="111">
         <f>SUM(F39:BB39)</f>
         <v>2.5</v>
       </c>
-      <c r="D39" s="112">
+      <c r="D39" s="111">
         <f>SUM(F40:BB40)</f>
         <v>0</v>
       </c>
-      <c r="E39" s="113">
+      <c r="E39" s="112">
         <f t="shared" ref="E39" si="2">(AVERAGE(C39,C40)-AVERAGE(D39,D40) )</f>
         <v>2.5</v>
       </c>
@@ -5134,8 +5161,8 @@
       <c r="BB39" s="32"/>
     </row>
     <row r="40" spans="1:54" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A40" s="171"/>
-      <c r="B40" s="173"/>
+      <c r="A40" s="169"/>
+      <c r="B40" s="171"/>
       <c r="C40" s="102"/>
       <c r="D40" s="102"/>
       <c r="E40" s="106"/>
@@ -5190,142 +5217,142 @@
       <c r="BB40" s="29"/>
     </row>
     <row r="41" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A41" s="176" t="b">
-        <v>0</v>
-      </c>
-      <c r="B41" s="178" t="s">
+      <c r="A41" s="174" t="b">
+        <v>0</v>
+      </c>
+      <c r="B41" s="176" t="s">
         <v>17</v>
       </c>
-      <c r="C41" s="180">
+      <c r="C41" s="178">
         <f>SUM(C43:C48)</f>
         <v>4.5</v>
       </c>
-      <c r="D41" s="180">
+      <c r="D41" s="178">
         <f>SUM(D43:D48)</f>
         <v>0</v>
       </c>
-      <c r="E41" s="180">
+      <c r="E41" s="178">
         <f>(C41-D41)</f>
         <v>4.5</v>
       </c>
-      <c r="F41" s="183"/>
-      <c r="G41" s="184"/>
-      <c r="H41" s="184"/>
-      <c r="I41" s="184"/>
-      <c r="J41" s="184"/>
-      <c r="K41" s="184"/>
-      <c r="L41" s="184"/>
-      <c r="M41" s="184"/>
-      <c r="N41" s="184"/>
-      <c r="O41" s="184"/>
-      <c r="P41" s="184"/>
-      <c r="Q41" s="184"/>
-      <c r="R41" s="184"/>
-      <c r="S41" s="184"/>
-      <c r="T41" s="184"/>
-      <c r="U41" s="184"/>
-      <c r="V41" s="184"/>
-      <c r="W41" s="184"/>
-      <c r="X41" s="184"/>
-      <c r="Y41" s="184"/>
-      <c r="Z41" s="184"/>
-      <c r="AA41" s="184"/>
-      <c r="AB41" s="184"/>
-      <c r="AC41" s="184"/>
-      <c r="AD41" s="184"/>
-      <c r="AE41" s="184"/>
-      <c r="AF41" s="184"/>
-      <c r="AG41" s="184"/>
-      <c r="AH41" s="184"/>
-      <c r="AI41" s="184"/>
-      <c r="AJ41" s="184"/>
-      <c r="AK41" s="184"/>
-      <c r="AL41" s="184"/>
-      <c r="AM41" s="184"/>
-      <c r="AN41" s="184"/>
-      <c r="AO41" s="184"/>
-      <c r="AP41" s="184"/>
-      <c r="AQ41" s="184"/>
-      <c r="AR41" s="184"/>
-      <c r="AS41" s="184"/>
-      <c r="AT41" s="184"/>
-      <c r="AU41" s="184"/>
-      <c r="AV41" s="184"/>
-      <c r="AW41" s="184"/>
-      <c r="AX41" s="184"/>
-      <c r="AY41" s="184"/>
-      <c r="AZ41" s="184"/>
-      <c r="BA41" s="184"/>
-      <c r="BB41" s="185"/>
+      <c r="F41" s="181"/>
+      <c r="G41" s="182"/>
+      <c r="H41" s="182"/>
+      <c r="I41" s="182"/>
+      <c r="J41" s="182"/>
+      <c r="K41" s="182"/>
+      <c r="L41" s="182"/>
+      <c r="M41" s="182"/>
+      <c r="N41" s="182"/>
+      <c r="O41" s="182"/>
+      <c r="P41" s="182"/>
+      <c r="Q41" s="182"/>
+      <c r="R41" s="182"/>
+      <c r="S41" s="182"/>
+      <c r="T41" s="182"/>
+      <c r="U41" s="182"/>
+      <c r="V41" s="182"/>
+      <c r="W41" s="182"/>
+      <c r="X41" s="182"/>
+      <c r="Y41" s="182"/>
+      <c r="Z41" s="182"/>
+      <c r="AA41" s="182"/>
+      <c r="AB41" s="182"/>
+      <c r="AC41" s="182"/>
+      <c r="AD41" s="182"/>
+      <c r="AE41" s="182"/>
+      <c r="AF41" s="182"/>
+      <c r="AG41" s="182"/>
+      <c r="AH41" s="182"/>
+      <c r="AI41" s="182"/>
+      <c r="AJ41" s="182"/>
+      <c r="AK41" s="182"/>
+      <c r="AL41" s="182"/>
+      <c r="AM41" s="182"/>
+      <c r="AN41" s="182"/>
+      <c r="AO41" s="182"/>
+      <c r="AP41" s="182"/>
+      <c r="AQ41" s="182"/>
+      <c r="AR41" s="182"/>
+      <c r="AS41" s="182"/>
+      <c r="AT41" s="182"/>
+      <c r="AU41" s="182"/>
+      <c r="AV41" s="182"/>
+      <c r="AW41" s="182"/>
+      <c r="AX41" s="182"/>
+      <c r="AY41" s="182"/>
+      <c r="AZ41" s="182"/>
+      <c r="BA41" s="182"/>
+      <c r="BB41" s="183"/>
     </row>
     <row r="42" spans="1:54" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A42" s="177"/>
-      <c r="B42" s="179"/>
-      <c r="C42" s="181"/>
-      <c r="D42" s="181"/>
-      <c r="E42" s="182"/>
-      <c r="F42" s="186"/>
-      <c r="G42" s="187"/>
-      <c r="H42" s="187"/>
-      <c r="I42" s="187"/>
-      <c r="J42" s="187"/>
-      <c r="K42" s="187"/>
-      <c r="L42" s="187"/>
-      <c r="M42" s="187"/>
-      <c r="N42" s="187"/>
-      <c r="O42" s="187"/>
-      <c r="P42" s="187"/>
-      <c r="Q42" s="187"/>
-      <c r="R42" s="187"/>
-      <c r="S42" s="187"/>
-      <c r="T42" s="187"/>
-      <c r="U42" s="187"/>
-      <c r="V42" s="187"/>
-      <c r="W42" s="187"/>
-      <c r="X42" s="187"/>
-      <c r="Y42" s="187"/>
-      <c r="Z42" s="187"/>
-      <c r="AA42" s="187"/>
-      <c r="AB42" s="187"/>
-      <c r="AC42" s="187"/>
-      <c r="AD42" s="187"/>
-      <c r="AE42" s="187"/>
-      <c r="AF42" s="187"/>
-      <c r="AG42" s="187"/>
-      <c r="AH42" s="187"/>
-      <c r="AI42" s="187"/>
-      <c r="AJ42" s="187"/>
-      <c r="AK42" s="187"/>
-      <c r="AL42" s="187"/>
-      <c r="AM42" s="187"/>
-      <c r="AN42" s="187"/>
-      <c r="AO42" s="187"/>
-      <c r="AP42" s="187"/>
-      <c r="AQ42" s="187"/>
-      <c r="AR42" s="187"/>
-      <c r="AS42" s="187"/>
-      <c r="AT42" s="187"/>
-      <c r="AU42" s="187"/>
-      <c r="AV42" s="187"/>
-      <c r="AW42" s="187"/>
-      <c r="AX42" s="187"/>
-      <c r="AY42" s="187"/>
-      <c r="AZ42" s="187"/>
-      <c r="BA42" s="187"/>
-      <c r="BB42" s="188"/>
+      <c r="A42" s="175"/>
+      <c r="B42" s="177"/>
+      <c r="C42" s="179"/>
+      <c r="D42" s="179"/>
+      <c r="E42" s="180"/>
+      <c r="F42" s="184"/>
+      <c r="G42" s="185"/>
+      <c r="H42" s="185"/>
+      <c r="I42" s="185"/>
+      <c r="J42" s="185"/>
+      <c r="K42" s="185"/>
+      <c r="L42" s="185"/>
+      <c r="M42" s="185"/>
+      <c r="N42" s="185"/>
+      <c r="O42" s="185"/>
+      <c r="P42" s="185"/>
+      <c r="Q42" s="185"/>
+      <c r="R42" s="185"/>
+      <c r="S42" s="185"/>
+      <c r="T42" s="185"/>
+      <c r="U42" s="185"/>
+      <c r="V42" s="185"/>
+      <c r="W42" s="185"/>
+      <c r="X42" s="185"/>
+      <c r="Y42" s="185"/>
+      <c r="Z42" s="185"/>
+      <c r="AA42" s="185"/>
+      <c r="AB42" s="185"/>
+      <c r="AC42" s="185"/>
+      <c r="AD42" s="185"/>
+      <c r="AE42" s="185"/>
+      <c r="AF42" s="185"/>
+      <c r="AG42" s="185"/>
+      <c r="AH42" s="185"/>
+      <c r="AI42" s="185"/>
+      <c r="AJ42" s="185"/>
+      <c r="AK42" s="185"/>
+      <c r="AL42" s="185"/>
+      <c r="AM42" s="185"/>
+      <c r="AN42" s="185"/>
+      <c r="AO42" s="185"/>
+      <c r="AP42" s="185"/>
+      <c r="AQ42" s="185"/>
+      <c r="AR42" s="185"/>
+      <c r="AS42" s="185"/>
+      <c r="AT42" s="185"/>
+      <c r="AU42" s="185"/>
+      <c r="AV42" s="185"/>
+      <c r="AW42" s="185"/>
+      <c r="AX42" s="185"/>
+      <c r="AY42" s="185"/>
+      <c r="AZ42" s="185"/>
+      <c r="BA42" s="185"/>
+      <c r="BB42" s="186"/>
     </row>
     <row r="43" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A43" s="202" t="b">
-        <v>0</v>
-      </c>
-      <c r="B43" s="204" t="s">
+      <c r="A43" s="200" t="b">
+        <v>0</v>
+      </c>
+      <c r="B43" s="202" t="s">
         <v>42</v>
       </c>
-      <c r="C43" s="112">
+      <c r="C43" s="111">
         <f>SUM(F43:BB43)</f>
         <v>1</v>
       </c>
-      <c r="D43" s="112">
+      <c r="D43" s="111">
         <f>SUM(F44:BB44)</f>
         <v>0</v>
       </c>
@@ -5386,8 +5413,8 @@
       <c r="BB43" s="40"/>
     </row>
     <row r="44" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A44" s="203"/>
-      <c r="B44" s="205"/>
+      <c r="A44" s="201"/>
+      <c r="B44" s="203"/>
       <c r="C44" s="102"/>
       <c r="D44" s="102"/>
       <c r="E44" s="106"/>
@@ -5442,21 +5469,21 @@
       <c r="BB44" s="29"/>
     </row>
     <row r="45" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A45" s="206" t="b">
-        <v>0</v>
-      </c>
-      <c r="B45" s="207" t="s">
+      <c r="A45" s="204" t="b">
+        <v>0</v>
+      </c>
+      <c r="B45" s="205" t="s">
         <v>44</v>
       </c>
-      <c r="C45" s="112">
+      <c r="C45" s="111">
         <f>SUM(F45:BB45)</f>
         <v>1</v>
       </c>
-      <c r="D45" s="112">
+      <c r="D45" s="111">
         <f>SUM(F46:BB46)</f>
         <v>0</v>
       </c>
-      <c r="E45" s="113">
+      <c r="E45" s="112">
         <f>(AVERAGE(C45,C46)-AVERAGE(D45,D46) )</f>
         <v>1</v>
       </c>
@@ -5513,11 +5540,11 @@
       <c r="BB45" s="32"/>
     </row>
     <row r="46" spans="1:54" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A46" s="203"/>
-      <c r="B46" s="205"/>
+      <c r="A46" s="201"/>
+      <c r="B46" s="203"/>
       <c r="C46" s="102"/>
       <c r="D46" s="102"/>
-      <c r="E46" s="145"/>
+      <c r="E46" s="143"/>
       <c r="F46" s="27"/>
       <c r="G46" s="28"/>
       <c r="H46" s="28"/>
@@ -5569,21 +5596,21 @@
       <c r="BB46" s="29"/>
     </row>
     <row r="47" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A47" s="206" t="b">
-        <v>0</v>
-      </c>
-      <c r="B47" s="207" t="s">
+      <c r="A47" s="204" t="b">
+        <v>0</v>
+      </c>
+      <c r="B47" s="205" t="s">
         <v>43</v>
       </c>
-      <c r="C47" s="112">
+      <c r="C47" s="111">
         <f>SUM(F47:BB47)</f>
         <v>2.5</v>
       </c>
-      <c r="D47" s="112">
+      <c r="D47" s="111">
         <f>SUM(F48:BB48)</f>
         <v>0</v>
       </c>
-      <c r="E47" s="113">
+      <c r="E47" s="112">
         <f>(AVERAGE(C47,C48)-AVERAGE(D47,D48) )</f>
         <v>2.5</v>
       </c>
@@ -5642,11 +5669,11 @@
       <c r="BB47" s="32"/>
     </row>
     <row r="48" spans="1:54" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A48" s="203"/>
-      <c r="B48" s="205"/>
+      <c r="A48" s="201"/>
+      <c r="B48" s="203"/>
       <c r="C48" s="102"/>
       <c r="D48" s="102"/>
-      <c r="E48" s="145"/>
+      <c r="E48" s="143"/>
       <c r="F48" s="27"/>
       <c r="G48" s="28"/>
       <c r="H48" s="28"/>
@@ -5698,142 +5725,142 @@
       <c r="BB48" s="29"/>
     </row>
     <row r="49" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A49" s="189" t="b">
-        <v>0</v>
-      </c>
-      <c r="B49" s="191" t="s">
+      <c r="A49" s="187" t="b">
+        <v>0</v>
+      </c>
+      <c r="B49" s="189" t="s">
         <v>18</v>
       </c>
-      <c r="C49" s="193">
+      <c r="C49" s="191">
         <f>SUM(C51:C66)</f>
         <v>23</v>
       </c>
-      <c r="D49" s="193">
+      <c r="D49" s="191">
         <f>SUM(D51:D66)</f>
         <v>0</v>
       </c>
-      <c r="E49" s="193">
+      <c r="E49" s="191">
         <f>(C49-D49)</f>
         <v>23</v>
       </c>
-      <c r="F49" s="196"/>
-      <c r="G49" s="197"/>
-      <c r="H49" s="197"/>
-      <c r="I49" s="197"/>
-      <c r="J49" s="197"/>
-      <c r="K49" s="197"/>
-      <c r="L49" s="197"/>
-      <c r="M49" s="197"/>
-      <c r="N49" s="197"/>
-      <c r="O49" s="197"/>
-      <c r="P49" s="197"/>
-      <c r="Q49" s="197"/>
-      <c r="R49" s="197"/>
-      <c r="S49" s="197"/>
-      <c r="T49" s="197"/>
-      <c r="U49" s="197"/>
-      <c r="V49" s="197"/>
-      <c r="W49" s="197"/>
-      <c r="X49" s="197"/>
-      <c r="Y49" s="197"/>
-      <c r="Z49" s="197"/>
-      <c r="AA49" s="197"/>
-      <c r="AB49" s="197"/>
-      <c r="AC49" s="197"/>
-      <c r="AD49" s="197"/>
-      <c r="AE49" s="197"/>
-      <c r="AF49" s="197"/>
-      <c r="AG49" s="197"/>
-      <c r="AH49" s="197"/>
-      <c r="AI49" s="197"/>
-      <c r="AJ49" s="197"/>
-      <c r="AK49" s="197"/>
-      <c r="AL49" s="197"/>
-      <c r="AM49" s="197"/>
-      <c r="AN49" s="197"/>
-      <c r="AO49" s="197"/>
-      <c r="AP49" s="197"/>
-      <c r="AQ49" s="197"/>
-      <c r="AR49" s="197"/>
-      <c r="AS49" s="197"/>
-      <c r="AT49" s="197"/>
-      <c r="AU49" s="197"/>
-      <c r="AV49" s="197"/>
-      <c r="AW49" s="197"/>
-      <c r="AX49" s="197"/>
-      <c r="AY49" s="197"/>
-      <c r="AZ49" s="197"/>
-      <c r="BA49" s="197"/>
-      <c r="BB49" s="198"/>
+      <c r="F49" s="194"/>
+      <c r="G49" s="195"/>
+      <c r="H49" s="195"/>
+      <c r="I49" s="195"/>
+      <c r="J49" s="195"/>
+      <c r="K49" s="195"/>
+      <c r="L49" s="195"/>
+      <c r="M49" s="195"/>
+      <c r="N49" s="195"/>
+      <c r="O49" s="195"/>
+      <c r="P49" s="195"/>
+      <c r="Q49" s="195"/>
+      <c r="R49" s="195"/>
+      <c r="S49" s="195"/>
+      <c r="T49" s="195"/>
+      <c r="U49" s="195"/>
+      <c r="V49" s="195"/>
+      <c r="W49" s="195"/>
+      <c r="X49" s="195"/>
+      <c r="Y49" s="195"/>
+      <c r="Z49" s="195"/>
+      <c r="AA49" s="195"/>
+      <c r="AB49" s="195"/>
+      <c r="AC49" s="195"/>
+      <c r="AD49" s="195"/>
+      <c r="AE49" s="195"/>
+      <c r="AF49" s="195"/>
+      <c r="AG49" s="195"/>
+      <c r="AH49" s="195"/>
+      <c r="AI49" s="195"/>
+      <c r="AJ49" s="195"/>
+      <c r="AK49" s="195"/>
+      <c r="AL49" s="195"/>
+      <c r="AM49" s="195"/>
+      <c r="AN49" s="195"/>
+      <c r="AO49" s="195"/>
+      <c r="AP49" s="195"/>
+      <c r="AQ49" s="195"/>
+      <c r="AR49" s="195"/>
+      <c r="AS49" s="195"/>
+      <c r="AT49" s="195"/>
+      <c r="AU49" s="195"/>
+      <c r="AV49" s="195"/>
+      <c r="AW49" s="195"/>
+      <c r="AX49" s="195"/>
+      <c r="AY49" s="195"/>
+      <c r="AZ49" s="195"/>
+      <c r="BA49" s="195"/>
+      <c r="BB49" s="196"/>
     </row>
     <row r="50" spans="1:54" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A50" s="190"/>
-      <c r="B50" s="192"/>
-      <c r="C50" s="194"/>
-      <c r="D50" s="194"/>
-      <c r="E50" s="195"/>
-      <c r="F50" s="199"/>
-      <c r="G50" s="200"/>
-      <c r="H50" s="200"/>
-      <c r="I50" s="200"/>
-      <c r="J50" s="200"/>
-      <c r="K50" s="200"/>
-      <c r="L50" s="200"/>
-      <c r="M50" s="200"/>
-      <c r="N50" s="200"/>
-      <c r="O50" s="200"/>
-      <c r="P50" s="200"/>
-      <c r="Q50" s="200"/>
-      <c r="R50" s="200"/>
-      <c r="S50" s="200"/>
-      <c r="T50" s="200"/>
-      <c r="U50" s="200"/>
-      <c r="V50" s="200"/>
-      <c r="W50" s="200"/>
-      <c r="X50" s="200"/>
-      <c r="Y50" s="200"/>
-      <c r="Z50" s="200"/>
-      <c r="AA50" s="200"/>
-      <c r="AB50" s="200"/>
-      <c r="AC50" s="200"/>
-      <c r="AD50" s="200"/>
-      <c r="AE50" s="200"/>
-      <c r="AF50" s="200"/>
-      <c r="AG50" s="200"/>
-      <c r="AH50" s="200"/>
-      <c r="AI50" s="200"/>
-      <c r="AJ50" s="200"/>
-      <c r="AK50" s="200"/>
-      <c r="AL50" s="200"/>
-      <c r="AM50" s="200"/>
-      <c r="AN50" s="200"/>
-      <c r="AO50" s="200"/>
-      <c r="AP50" s="200"/>
-      <c r="AQ50" s="200"/>
-      <c r="AR50" s="200"/>
-      <c r="AS50" s="200"/>
-      <c r="AT50" s="200"/>
-      <c r="AU50" s="200"/>
-      <c r="AV50" s="200"/>
-      <c r="AW50" s="200"/>
-      <c r="AX50" s="200"/>
-      <c r="AY50" s="200"/>
-      <c r="AZ50" s="200"/>
-      <c r="BA50" s="200"/>
-      <c r="BB50" s="201"/>
+      <c r="A50" s="188"/>
+      <c r="B50" s="190"/>
+      <c r="C50" s="192"/>
+      <c r="D50" s="192"/>
+      <c r="E50" s="193"/>
+      <c r="F50" s="197"/>
+      <c r="G50" s="198"/>
+      <c r="H50" s="198"/>
+      <c r="I50" s="198"/>
+      <c r="J50" s="198"/>
+      <c r="K50" s="198"/>
+      <c r="L50" s="198"/>
+      <c r="M50" s="198"/>
+      <c r="N50" s="198"/>
+      <c r="O50" s="198"/>
+      <c r="P50" s="198"/>
+      <c r="Q50" s="198"/>
+      <c r="R50" s="198"/>
+      <c r="S50" s="198"/>
+      <c r="T50" s="198"/>
+      <c r="U50" s="198"/>
+      <c r="V50" s="198"/>
+      <c r="W50" s="198"/>
+      <c r="X50" s="198"/>
+      <c r="Y50" s="198"/>
+      <c r="Z50" s="198"/>
+      <c r="AA50" s="198"/>
+      <c r="AB50" s="198"/>
+      <c r="AC50" s="198"/>
+      <c r="AD50" s="198"/>
+      <c r="AE50" s="198"/>
+      <c r="AF50" s="198"/>
+      <c r="AG50" s="198"/>
+      <c r="AH50" s="198"/>
+      <c r="AI50" s="198"/>
+      <c r="AJ50" s="198"/>
+      <c r="AK50" s="198"/>
+      <c r="AL50" s="198"/>
+      <c r="AM50" s="198"/>
+      <c r="AN50" s="198"/>
+      <c r="AO50" s="198"/>
+      <c r="AP50" s="198"/>
+      <c r="AQ50" s="198"/>
+      <c r="AR50" s="198"/>
+      <c r="AS50" s="198"/>
+      <c r="AT50" s="198"/>
+      <c r="AU50" s="198"/>
+      <c r="AV50" s="198"/>
+      <c r="AW50" s="198"/>
+      <c r="AX50" s="198"/>
+      <c r="AY50" s="198"/>
+      <c r="AZ50" s="198"/>
+      <c r="BA50" s="198"/>
+      <c r="BB50" s="199"/>
     </row>
     <row r="51" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A51" s="208" t="b">
-        <v>0</v>
-      </c>
-      <c r="B51" s="210" t="s">
-        <v>56</v>
-      </c>
-      <c r="C51" s="112">
+      <c r="A51" s="206" t="b">
+        <v>0</v>
+      </c>
+      <c r="B51" s="208" t="s">
+        <v>55</v>
+      </c>
+      <c r="C51" s="111">
         <f>SUM(F51:BB51)</f>
         <v>3</v>
       </c>
-      <c r="D51" s="112">
+      <c r="D51" s="111">
         <f>SUM(F52:BB52)</f>
         <v>0</v>
       </c>
@@ -5898,8 +5925,8 @@
       <c r="BB51" s="40"/>
     </row>
     <row r="52" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A52" s="209"/>
-      <c r="B52" s="211"/>
+      <c r="A52" s="207"/>
+      <c r="B52" s="209"/>
       <c r="C52" s="102"/>
       <c r="D52" s="102"/>
       <c r="E52" s="106"/>
@@ -5954,21 +5981,21 @@
       <c r="BB52" s="29"/>
     </row>
     <row r="53" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A53" s="212" t="b">
-        <v>0</v>
-      </c>
-      <c r="B53" s="210" t="s">
-        <v>57</v>
-      </c>
-      <c r="C53" s="112">
+      <c r="A53" s="210" t="b">
+        <v>0</v>
+      </c>
+      <c r="B53" s="208" t="s">
+        <v>56</v>
+      </c>
+      <c r="C53" s="111">
         <f>SUM(F53:BB53)</f>
         <v>1.5</v>
       </c>
-      <c r="D53" s="112">
+      <c r="D53" s="111">
         <f>SUM(F54:BB54)</f>
         <v>0</v>
       </c>
-      <c r="E53" s="113">
+      <c r="E53" s="112">
         <f t="shared" ref="E53:E65" si="3">(AVERAGE(C53,C54)-AVERAGE(D53,D54) )</f>
         <v>1.5</v>
       </c>
@@ -6025,8 +6052,8 @@
       <c r="BB53" s="32"/>
     </row>
     <row r="54" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A54" s="209"/>
-      <c r="B54" s="211"/>
+      <c r="A54" s="207"/>
+      <c r="B54" s="209"/>
       <c r="C54" s="102"/>
       <c r="D54" s="102"/>
       <c r="E54" s="106"/>
@@ -6081,21 +6108,21 @@
       <c r="BB54" s="29"/>
     </row>
     <row r="55" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A55" s="212" t="b">
-        <v>0</v>
-      </c>
-      <c r="B55" s="210" t="s">
-        <v>59</v>
-      </c>
-      <c r="C55" s="112">
+      <c r="A55" s="210" t="b">
+        <v>0</v>
+      </c>
+      <c r="B55" s="208" t="s">
+        <v>58</v>
+      </c>
+      <c r="C55" s="111">
         <f>SUM(F55:BB55)</f>
         <v>1.5</v>
       </c>
-      <c r="D55" s="112">
+      <c r="D55" s="111">
         <f>SUM(F56:BB56)</f>
         <v>0</v>
       </c>
-      <c r="E55" s="113">
+      <c r="E55" s="112">
         <f t="shared" si="3"/>
         <v>1.5</v>
       </c>
@@ -6152,8 +6179,8 @@
       <c r="BB55" s="32"/>
     </row>
     <row r="56" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A56" s="209"/>
-      <c r="B56" s="211"/>
+      <c r="A56" s="207"/>
+      <c r="B56" s="209"/>
       <c r="C56" s="102"/>
       <c r="D56" s="102"/>
       <c r="E56" s="106"/>
@@ -6208,21 +6235,21 @@
       <c r="BB56" s="29"/>
     </row>
     <row r="57" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A57" s="212" t="b">
-        <v>0</v>
-      </c>
-      <c r="B57" s="210" t="s">
-        <v>58</v>
-      </c>
-      <c r="C57" s="112">
+      <c r="A57" s="210" t="b">
+        <v>0</v>
+      </c>
+      <c r="B57" s="208" t="s">
+        <v>57</v>
+      </c>
+      <c r="C57" s="111">
         <f>SUM(F57:BB57)</f>
         <v>5.5</v>
       </c>
-      <c r="D57" s="112">
+      <c r="D57" s="111">
         <f>SUM(F58:BB58)</f>
         <v>0</v>
       </c>
-      <c r="E57" s="113">
+      <c r="E57" s="112">
         <f t="shared" si="3"/>
         <v>5.5</v>
       </c>
@@ -6289,8 +6316,8 @@
       <c r="BB57" s="32"/>
     </row>
     <row r="58" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A58" s="209"/>
-      <c r="B58" s="211"/>
+      <c r="A58" s="207"/>
+      <c r="B58" s="209"/>
       <c r="C58" s="102"/>
       <c r="D58" s="102"/>
       <c r="E58" s="106"/>
@@ -6345,21 +6372,21 @@
       <c r="BB58" s="29"/>
     </row>
     <row r="59" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A59" s="212" t="b">
-        <v>0</v>
-      </c>
-      <c r="B59" s="210" t="s">
-        <v>60</v>
-      </c>
-      <c r="C59" s="112">
+      <c r="A59" s="210" t="b">
+        <v>0</v>
+      </c>
+      <c r="B59" s="208" t="s">
+        <v>59</v>
+      </c>
+      <c r="C59" s="111">
         <f>SUM(F59:BB59)</f>
         <v>4</v>
       </c>
-      <c r="D59" s="112">
+      <c r="D59" s="111">
         <f>SUM(F60:BB60)</f>
         <v>0</v>
       </c>
-      <c r="E59" s="113">
+      <c r="E59" s="112">
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
@@ -6422,8 +6449,8 @@
       <c r="BB59" s="32"/>
     </row>
     <row r="60" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A60" s="209"/>
-      <c r="B60" s="211"/>
+      <c r="A60" s="207"/>
+      <c r="B60" s="209"/>
       <c r="C60" s="102"/>
       <c r="D60" s="102"/>
       <c r="E60" s="106"/>
@@ -6478,21 +6505,21 @@
       <c r="BB60" s="29"/>
     </row>
     <row r="61" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A61" s="212" t="b">
-        <v>0</v>
-      </c>
-      <c r="B61" s="210" t="s">
-        <v>61</v>
-      </c>
-      <c r="C61" s="112">
+      <c r="A61" s="210" t="b">
+        <v>0</v>
+      </c>
+      <c r="B61" s="208" t="s">
+        <v>60</v>
+      </c>
+      <c r="C61" s="111">
         <f>SUM(F61:BB61)</f>
         <v>1.5</v>
       </c>
-      <c r="D61" s="112">
+      <c r="D61" s="111">
         <f>SUM(F62:BB62)</f>
         <v>0</v>
       </c>
-      <c r="E61" s="113">
+      <c r="E61" s="112">
         <f t="shared" si="3"/>
         <v>1.5</v>
       </c>
@@ -6549,8 +6576,8 @@
       <c r="BB61" s="32"/>
     </row>
     <row r="62" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A62" s="209"/>
-      <c r="B62" s="211"/>
+      <c r="A62" s="207"/>
+      <c r="B62" s="209"/>
       <c r="C62" s="102"/>
       <c r="D62" s="102"/>
       <c r="E62" s="106"/>
@@ -6605,21 +6632,21 @@
       <c r="BB62" s="29"/>
     </row>
     <row r="63" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A63" s="212" t="b">
-        <v>0</v>
-      </c>
-      <c r="B63" s="213" t="s">
-        <v>62</v>
-      </c>
-      <c r="C63" s="112">
+      <c r="A63" s="210" t="b">
+        <v>0</v>
+      </c>
+      <c r="B63" s="211" t="s">
+        <v>61</v>
+      </c>
+      <c r="C63" s="111">
         <f>SUM(F63:BB63)</f>
         <v>1.5</v>
       </c>
-      <c r="D63" s="112">
+      <c r="D63" s="111">
         <f>SUM(F64:BB64)</f>
         <v>0</v>
       </c>
-      <c r="E63" s="113">
+      <c r="E63" s="112">
         <f t="shared" si="3"/>
         <v>1.5</v>
       </c>
@@ -6676,8 +6703,8 @@
       <c r="BB63" s="32"/>
     </row>
     <row r="64" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A64" s="209"/>
-      <c r="B64" s="214"/>
+      <c r="A64" s="207"/>
+      <c r="B64" s="212"/>
       <c r="C64" s="102"/>
       <c r="D64" s="102"/>
       <c r="E64" s="106"/>
@@ -6732,21 +6759,21 @@
       <c r="BB64" s="29"/>
     </row>
     <row r="65" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A65" s="212" t="b">
-        <v>0</v>
-      </c>
-      <c r="B65" s="215" t="s">
-        <v>64</v>
-      </c>
-      <c r="C65" s="112">
+      <c r="A65" s="210" t="b">
+        <v>0</v>
+      </c>
+      <c r="B65" s="213" t="s">
+        <v>63</v>
+      </c>
+      <c r="C65" s="111">
         <f>SUM(F65:BB65)</f>
         <v>4.5</v>
       </c>
-      <c r="D65" s="112">
+      <c r="D65" s="111">
         <f>SUM(F66:BB66)</f>
         <v>0</v>
       </c>
-      <c r="E65" s="113">
+      <c r="E65" s="112">
         <f t="shared" si="3"/>
         <v>4.5</v>
       </c>
@@ -6764,7 +6791,7 @@
       <c r="Q65" s="58"/>
       <c r="R65" s="58"/>
       <c r="S65" s="58"/>
-      <c r="T65" s="278"/>
+      <c r="T65" s="276"/>
       <c r="U65" s="30"/>
       <c r="V65" s="31"/>
       <c r="W65" s="31"/>
@@ -6807,8 +6834,8 @@
       <c r="BB65" s="32"/>
     </row>
     <row r="66" spans="1:54" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A66" s="209"/>
-      <c r="B66" s="211"/>
+      <c r="A66" s="207"/>
+      <c r="B66" s="209"/>
       <c r="C66" s="102"/>
       <c r="D66" s="102"/>
       <c r="E66" s="106"/>
@@ -6863,142 +6890,142 @@
       <c r="BB66" s="29"/>
     </row>
     <row r="67" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A67" s="226" t="b">
-        <v>0</v>
-      </c>
-      <c r="B67" s="228" t="s">
+      <c r="A67" s="224" t="b">
+        <v>0</v>
+      </c>
+      <c r="B67" s="226" t="s">
         <v>19</v>
       </c>
-      <c r="C67" s="230">
+      <c r="C67" s="228">
         <f>SUM(C69:C74)</f>
         <v>3.5</v>
       </c>
-      <c r="D67" s="230">
+      <c r="D67" s="228">
         <f>SUM(D69:D74)</f>
         <v>0</v>
       </c>
-      <c r="E67" s="230">
+      <c r="E67" s="228">
         <f>(C67-D67)</f>
         <v>3.5</v>
       </c>
-      <c r="F67" s="216"/>
-      <c r="G67" s="217"/>
-      <c r="H67" s="217"/>
-      <c r="I67" s="217"/>
-      <c r="J67" s="217"/>
-      <c r="K67" s="217"/>
-      <c r="L67" s="217"/>
-      <c r="M67" s="217"/>
-      <c r="N67" s="217"/>
-      <c r="O67" s="217"/>
-      <c r="P67" s="217"/>
-      <c r="Q67" s="217"/>
-      <c r="R67" s="217"/>
-      <c r="S67" s="217"/>
-      <c r="T67" s="217"/>
-      <c r="U67" s="217"/>
-      <c r="V67" s="217"/>
-      <c r="W67" s="217"/>
-      <c r="X67" s="217"/>
-      <c r="Y67" s="217"/>
-      <c r="Z67" s="217"/>
-      <c r="AA67" s="217"/>
-      <c r="AB67" s="217"/>
-      <c r="AC67" s="217"/>
-      <c r="AD67" s="217"/>
-      <c r="AE67" s="217"/>
-      <c r="AF67" s="217"/>
-      <c r="AG67" s="217"/>
-      <c r="AH67" s="217"/>
-      <c r="AI67" s="217"/>
-      <c r="AJ67" s="217"/>
-      <c r="AK67" s="217"/>
-      <c r="AL67" s="217"/>
-      <c r="AM67" s="217"/>
-      <c r="AN67" s="217"/>
-      <c r="AO67" s="217"/>
-      <c r="AP67" s="217"/>
-      <c r="AQ67" s="217"/>
-      <c r="AR67" s="217"/>
-      <c r="AS67" s="217"/>
-      <c r="AT67" s="217"/>
-      <c r="AU67" s="217"/>
-      <c r="AV67" s="217"/>
-      <c r="AW67" s="217"/>
-      <c r="AX67" s="217"/>
-      <c r="AY67" s="217"/>
-      <c r="AZ67" s="217"/>
-      <c r="BA67" s="217"/>
-      <c r="BB67" s="218"/>
+      <c r="F67" s="214"/>
+      <c r="G67" s="215"/>
+      <c r="H67" s="215"/>
+      <c r="I67" s="215"/>
+      <c r="J67" s="215"/>
+      <c r="K67" s="215"/>
+      <c r="L67" s="215"/>
+      <c r="M67" s="215"/>
+      <c r="N67" s="215"/>
+      <c r="O67" s="215"/>
+      <c r="P67" s="215"/>
+      <c r="Q67" s="215"/>
+      <c r="R67" s="215"/>
+      <c r="S67" s="215"/>
+      <c r="T67" s="215"/>
+      <c r="U67" s="215"/>
+      <c r="V67" s="215"/>
+      <c r="W67" s="215"/>
+      <c r="X67" s="215"/>
+      <c r="Y67" s="215"/>
+      <c r="Z67" s="215"/>
+      <c r="AA67" s="215"/>
+      <c r="AB67" s="215"/>
+      <c r="AC67" s="215"/>
+      <c r="AD67" s="215"/>
+      <c r="AE67" s="215"/>
+      <c r="AF67" s="215"/>
+      <c r="AG67" s="215"/>
+      <c r="AH67" s="215"/>
+      <c r="AI67" s="215"/>
+      <c r="AJ67" s="215"/>
+      <c r="AK67" s="215"/>
+      <c r="AL67" s="215"/>
+      <c r="AM67" s="215"/>
+      <c r="AN67" s="215"/>
+      <c r="AO67" s="215"/>
+      <c r="AP67" s="215"/>
+      <c r="AQ67" s="215"/>
+      <c r="AR67" s="215"/>
+      <c r="AS67" s="215"/>
+      <c r="AT67" s="215"/>
+      <c r="AU67" s="215"/>
+      <c r="AV67" s="215"/>
+      <c r="AW67" s="215"/>
+      <c r="AX67" s="215"/>
+      <c r="AY67" s="215"/>
+      <c r="AZ67" s="215"/>
+      <c r="BA67" s="215"/>
+      <c r="BB67" s="216"/>
     </row>
     <row r="68" spans="1:54" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A68" s="227"/>
-      <c r="B68" s="229"/>
-      <c r="C68" s="231"/>
-      <c r="D68" s="231"/>
-      <c r="E68" s="232"/>
-      <c r="F68" s="219"/>
-      <c r="G68" s="220"/>
-      <c r="H68" s="220"/>
-      <c r="I68" s="220"/>
-      <c r="J68" s="220"/>
-      <c r="K68" s="220"/>
-      <c r="L68" s="220"/>
-      <c r="M68" s="220"/>
-      <c r="N68" s="220"/>
-      <c r="O68" s="220"/>
-      <c r="P68" s="220"/>
-      <c r="Q68" s="220"/>
-      <c r="R68" s="220"/>
-      <c r="S68" s="220"/>
-      <c r="T68" s="220"/>
-      <c r="U68" s="220"/>
-      <c r="V68" s="220"/>
-      <c r="W68" s="220"/>
-      <c r="X68" s="220"/>
-      <c r="Y68" s="220"/>
-      <c r="Z68" s="220"/>
-      <c r="AA68" s="220"/>
-      <c r="AB68" s="220"/>
-      <c r="AC68" s="220"/>
-      <c r="AD68" s="220"/>
-      <c r="AE68" s="220"/>
-      <c r="AF68" s="220"/>
-      <c r="AG68" s="220"/>
-      <c r="AH68" s="220"/>
-      <c r="AI68" s="220"/>
-      <c r="AJ68" s="220"/>
-      <c r="AK68" s="220"/>
-      <c r="AL68" s="220"/>
-      <c r="AM68" s="220"/>
-      <c r="AN68" s="220"/>
-      <c r="AO68" s="220"/>
-      <c r="AP68" s="220"/>
-      <c r="AQ68" s="220"/>
-      <c r="AR68" s="220"/>
-      <c r="AS68" s="220"/>
-      <c r="AT68" s="220"/>
-      <c r="AU68" s="220"/>
-      <c r="AV68" s="220"/>
-      <c r="AW68" s="220"/>
-      <c r="AX68" s="220"/>
-      <c r="AY68" s="220"/>
-      <c r="AZ68" s="220"/>
-      <c r="BA68" s="220"/>
-      <c r="BB68" s="221"/>
+      <c r="A68" s="225"/>
+      <c r="B68" s="227"/>
+      <c r="C68" s="229"/>
+      <c r="D68" s="229"/>
+      <c r="E68" s="230"/>
+      <c r="F68" s="217"/>
+      <c r="G68" s="218"/>
+      <c r="H68" s="218"/>
+      <c r="I68" s="218"/>
+      <c r="J68" s="218"/>
+      <c r="K68" s="218"/>
+      <c r="L68" s="218"/>
+      <c r="M68" s="218"/>
+      <c r="N68" s="218"/>
+      <c r="O68" s="218"/>
+      <c r="P68" s="218"/>
+      <c r="Q68" s="218"/>
+      <c r="R68" s="218"/>
+      <c r="S68" s="218"/>
+      <c r="T68" s="218"/>
+      <c r="U68" s="218"/>
+      <c r="V68" s="218"/>
+      <c r="W68" s="218"/>
+      <c r="X68" s="218"/>
+      <c r="Y68" s="218"/>
+      <c r="Z68" s="218"/>
+      <c r="AA68" s="218"/>
+      <c r="AB68" s="218"/>
+      <c r="AC68" s="218"/>
+      <c r="AD68" s="218"/>
+      <c r="AE68" s="218"/>
+      <c r="AF68" s="218"/>
+      <c r="AG68" s="218"/>
+      <c r="AH68" s="218"/>
+      <c r="AI68" s="218"/>
+      <c r="AJ68" s="218"/>
+      <c r="AK68" s="218"/>
+      <c r="AL68" s="218"/>
+      <c r="AM68" s="218"/>
+      <c r="AN68" s="218"/>
+      <c r="AO68" s="218"/>
+      <c r="AP68" s="218"/>
+      <c r="AQ68" s="218"/>
+      <c r="AR68" s="218"/>
+      <c r="AS68" s="218"/>
+      <c r="AT68" s="218"/>
+      <c r="AU68" s="218"/>
+      <c r="AV68" s="218"/>
+      <c r="AW68" s="218"/>
+      <c r="AX68" s="218"/>
+      <c r="AY68" s="218"/>
+      <c r="AZ68" s="218"/>
+      <c r="BA68" s="218"/>
+      <c r="BB68" s="219"/>
     </row>
     <row r="69" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A69" s="222" t="b">
-        <v>0</v>
-      </c>
-      <c r="B69" s="224" t="s">
+      <c r="A69" s="220" t="b">
+        <v>0</v>
+      </c>
+      <c r="B69" s="222" t="s">
         <v>45</v>
       </c>
-      <c r="C69" s="112">
+      <c r="C69" s="111">
         <f>SUM(F69:BB69)</f>
         <v>1.5</v>
       </c>
-      <c r="D69" s="112">
+      <c r="D69" s="111">
         <f>SUM(F70:BB70)</f>
         <v>0</v>
       </c>
@@ -7059,8 +7086,8 @@
       <c r="BB69" s="32"/>
     </row>
     <row r="70" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A70" s="223"/>
-      <c r="B70" s="225"/>
+      <c r="A70" s="221"/>
+      <c r="B70" s="223"/>
       <c r="C70" s="102"/>
       <c r="D70" s="102"/>
       <c r="E70" s="106"/>
@@ -7115,21 +7142,21 @@
       <c r="BB70" s="29"/>
     </row>
     <row r="71" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A71" s="244" t="b">
-        <v>0</v>
-      </c>
-      <c r="B71" s="245" t="s">
+      <c r="A71" s="242" t="b">
+        <v>0</v>
+      </c>
+      <c r="B71" s="243" t="s">
         <v>46</v>
       </c>
-      <c r="C71" s="112">
+      <c r="C71" s="111">
         <f>SUM(F71:BB71)</f>
         <v>1</v>
       </c>
-      <c r="D71" s="112">
+      <c r="D71" s="111">
         <f>SUM(F72:BB72)</f>
         <v>0</v>
       </c>
-      <c r="E71" s="113">
+      <c r="E71" s="112">
         <f t="shared" ref="E71" si="4">(AVERAGE(C71,C72)-AVERAGE(D71,D72) )</f>
         <v>1</v>
       </c>
@@ -7186,8 +7213,8 @@
       <c r="BB71" s="32"/>
     </row>
     <row r="72" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A72" s="223"/>
-      <c r="B72" s="246"/>
+      <c r="A72" s="221"/>
+      <c r="B72" s="244"/>
       <c r="C72" s="102"/>
       <c r="D72" s="102"/>
       <c r="E72" s="106"/>
@@ -7242,21 +7269,21 @@
       <c r="BB72" s="29"/>
     </row>
     <row r="73" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A73" s="247" t="b">
-        <v>0</v>
-      </c>
-      <c r="B73" s="248" t="s">
+      <c r="A73" s="245" t="b">
+        <v>0</v>
+      </c>
+      <c r="B73" s="246" t="s">
         <v>47</v>
       </c>
-      <c r="C73" s="112">
+      <c r="C73" s="111">
         <f>SUM(F73:BB73)</f>
         <v>1</v>
       </c>
-      <c r="D73" s="112">
+      <c r="D73" s="111">
         <f>SUM(F74:BB74)</f>
         <v>0</v>
       </c>
-      <c r="E73" s="113">
+      <c r="E73" s="112">
         <f>(AVERAGE(C73,C74)-AVERAGE(D73,D74) )</f>
         <v>1</v>
       </c>
@@ -7313,11 +7340,11 @@
       <c r="BB73" s="26"/>
     </row>
     <row r="74" spans="1:54" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A74" s="247"/>
-      <c r="B74" s="249"/>
+      <c r="A74" s="245"/>
+      <c r="B74" s="247"/>
       <c r="C74" s="102"/>
       <c r="D74" s="102"/>
-      <c r="E74" s="145"/>
+      <c r="E74" s="143"/>
       <c r="F74" s="25"/>
       <c r="G74" s="58"/>
       <c r="H74" s="58"/>
@@ -7369,142 +7396,142 @@
       <c r="BB74" s="26"/>
     </row>
     <row r="75" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A75" s="233" t="b">
-        <v>0</v>
-      </c>
-      <c r="B75" s="235" t="s">
+      <c r="A75" s="231" t="b">
+        <v>0</v>
+      </c>
+      <c r="B75" s="233" t="s">
         <v>20</v>
       </c>
-      <c r="C75" s="128">
+      <c r="C75" s="127">
         <f>SUM(C77:C86)</f>
         <v>11</v>
       </c>
-      <c r="D75" s="128">
+      <c r="D75" s="127">
         <f>SUM(D77:D86)</f>
         <v>0</v>
       </c>
-      <c r="E75" s="128">
+      <c r="E75" s="127">
         <f>(C75-D75)</f>
         <v>11</v>
       </c>
-      <c r="F75" s="238"/>
-      <c r="G75" s="239"/>
-      <c r="H75" s="239"/>
-      <c r="I75" s="239"/>
-      <c r="J75" s="239"/>
-      <c r="K75" s="239"/>
-      <c r="L75" s="239"/>
-      <c r="M75" s="239"/>
-      <c r="N75" s="239"/>
-      <c r="O75" s="239"/>
-      <c r="P75" s="239"/>
-      <c r="Q75" s="239"/>
-      <c r="R75" s="239"/>
-      <c r="S75" s="239"/>
-      <c r="T75" s="239"/>
-      <c r="U75" s="239"/>
-      <c r="V75" s="239"/>
-      <c r="W75" s="239"/>
-      <c r="X75" s="239"/>
-      <c r="Y75" s="239"/>
-      <c r="Z75" s="239"/>
-      <c r="AA75" s="239"/>
-      <c r="AB75" s="239"/>
-      <c r="AC75" s="239"/>
-      <c r="AD75" s="239"/>
-      <c r="AE75" s="239"/>
-      <c r="AF75" s="239"/>
-      <c r="AG75" s="239"/>
-      <c r="AH75" s="239"/>
-      <c r="AI75" s="239"/>
-      <c r="AJ75" s="239"/>
-      <c r="AK75" s="239"/>
-      <c r="AL75" s="239"/>
-      <c r="AM75" s="239"/>
-      <c r="AN75" s="239"/>
-      <c r="AO75" s="239"/>
-      <c r="AP75" s="239"/>
-      <c r="AQ75" s="239"/>
-      <c r="AR75" s="239"/>
-      <c r="AS75" s="239"/>
-      <c r="AT75" s="239"/>
-      <c r="AU75" s="239"/>
-      <c r="AV75" s="239"/>
-      <c r="AW75" s="239"/>
-      <c r="AX75" s="239"/>
-      <c r="AY75" s="239"/>
-      <c r="AZ75" s="239"/>
-      <c r="BA75" s="239"/>
-      <c r="BB75" s="240"/>
+      <c r="F75" s="236"/>
+      <c r="G75" s="237"/>
+      <c r="H75" s="237"/>
+      <c r="I75" s="237"/>
+      <c r="J75" s="237"/>
+      <c r="K75" s="237"/>
+      <c r="L75" s="237"/>
+      <c r="M75" s="237"/>
+      <c r="N75" s="237"/>
+      <c r="O75" s="237"/>
+      <c r="P75" s="237"/>
+      <c r="Q75" s="237"/>
+      <c r="R75" s="237"/>
+      <c r="S75" s="237"/>
+      <c r="T75" s="237"/>
+      <c r="U75" s="237"/>
+      <c r="V75" s="237"/>
+      <c r="W75" s="237"/>
+      <c r="X75" s="237"/>
+      <c r="Y75" s="237"/>
+      <c r="Z75" s="237"/>
+      <c r="AA75" s="237"/>
+      <c r="AB75" s="237"/>
+      <c r="AC75" s="237"/>
+      <c r="AD75" s="237"/>
+      <c r="AE75" s="237"/>
+      <c r="AF75" s="237"/>
+      <c r="AG75" s="237"/>
+      <c r="AH75" s="237"/>
+      <c r="AI75" s="237"/>
+      <c r="AJ75" s="237"/>
+      <c r="AK75" s="237"/>
+      <c r="AL75" s="237"/>
+      <c r="AM75" s="237"/>
+      <c r="AN75" s="237"/>
+      <c r="AO75" s="237"/>
+      <c r="AP75" s="237"/>
+      <c r="AQ75" s="237"/>
+      <c r="AR75" s="237"/>
+      <c r="AS75" s="237"/>
+      <c r="AT75" s="237"/>
+      <c r="AU75" s="237"/>
+      <c r="AV75" s="237"/>
+      <c r="AW75" s="237"/>
+      <c r="AX75" s="237"/>
+      <c r="AY75" s="237"/>
+      <c r="AZ75" s="237"/>
+      <c r="BA75" s="237"/>
+      <c r="BB75" s="238"/>
     </row>
     <row r="76" spans="1:54" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A76" s="234"/>
-      <c r="B76" s="236"/>
-      <c r="C76" s="237"/>
-      <c r="D76" s="237"/>
-      <c r="E76" s="129"/>
-      <c r="F76" s="241"/>
-      <c r="G76" s="242"/>
-      <c r="H76" s="242"/>
-      <c r="I76" s="242"/>
-      <c r="J76" s="242"/>
-      <c r="K76" s="242"/>
-      <c r="L76" s="242"/>
-      <c r="M76" s="242"/>
-      <c r="N76" s="242"/>
-      <c r="O76" s="242"/>
-      <c r="P76" s="242"/>
-      <c r="Q76" s="242"/>
-      <c r="R76" s="242"/>
-      <c r="S76" s="242"/>
-      <c r="T76" s="242"/>
-      <c r="U76" s="242"/>
-      <c r="V76" s="242"/>
-      <c r="W76" s="242"/>
-      <c r="X76" s="242"/>
-      <c r="Y76" s="242"/>
-      <c r="Z76" s="242"/>
-      <c r="AA76" s="242"/>
-      <c r="AB76" s="242"/>
-      <c r="AC76" s="242"/>
-      <c r="AD76" s="242"/>
-      <c r="AE76" s="242"/>
-      <c r="AF76" s="242"/>
-      <c r="AG76" s="242"/>
-      <c r="AH76" s="242"/>
-      <c r="AI76" s="242"/>
-      <c r="AJ76" s="242"/>
-      <c r="AK76" s="242"/>
-      <c r="AL76" s="242"/>
-      <c r="AM76" s="242"/>
-      <c r="AN76" s="242"/>
-      <c r="AO76" s="242"/>
-      <c r="AP76" s="242"/>
-      <c r="AQ76" s="242"/>
-      <c r="AR76" s="242"/>
-      <c r="AS76" s="242"/>
-      <c r="AT76" s="242"/>
-      <c r="AU76" s="242"/>
-      <c r="AV76" s="242"/>
-      <c r="AW76" s="242"/>
-      <c r="AX76" s="242"/>
-      <c r="AY76" s="242"/>
-      <c r="AZ76" s="242"/>
-      <c r="BA76" s="242"/>
-      <c r="BB76" s="243"/>
+      <c r="A76" s="232"/>
+      <c r="B76" s="234"/>
+      <c r="C76" s="235"/>
+      <c r="D76" s="235"/>
+      <c r="E76" s="128"/>
+      <c r="F76" s="239"/>
+      <c r="G76" s="240"/>
+      <c r="H76" s="240"/>
+      <c r="I76" s="240"/>
+      <c r="J76" s="240"/>
+      <c r="K76" s="240"/>
+      <c r="L76" s="240"/>
+      <c r="M76" s="240"/>
+      <c r="N76" s="240"/>
+      <c r="O76" s="240"/>
+      <c r="P76" s="240"/>
+      <c r="Q76" s="240"/>
+      <c r="R76" s="240"/>
+      <c r="S76" s="240"/>
+      <c r="T76" s="240"/>
+      <c r="U76" s="240"/>
+      <c r="V76" s="240"/>
+      <c r="W76" s="240"/>
+      <c r="X76" s="240"/>
+      <c r="Y76" s="240"/>
+      <c r="Z76" s="240"/>
+      <c r="AA76" s="240"/>
+      <c r="AB76" s="240"/>
+      <c r="AC76" s="240"/>
+      <c r="AD76" s="240"/>
+      <c r="AE76" s="240"/>
+      <c r="AF76" s="240"/>
+      <c r="AG76" s="240"/>
+      <c r="AH76" s="240"/>
+      <c r="AI76" s="240"/>
+      <c r="AJ76" s="240"/>
+      <c r="AK76" s="240"/>
+      <c r="AL76" s="240"/>
+      <c r="AM76" s="240"/>
+      <c r="AN76" s="240"/>
+      <c r="AO76" s="240"/>
+      <c r="AP76" s="240"/>
+      <c r="AQ76" s="240"/>
+      <c r="AR76" s="240"/>
+      <c r="AS76" s="240"/>
+      <c r="AT76" s="240"/>
+      <c r="AU76" s="240"/>
+      <c r="AV76" s="240"/>
+      <c r="AW76" s="240"/>
+      <c r="AX76" s="240"/>
+      <c r="AY76" s="240"/>
+      <c r="AZ76" s="240"/>
+      <c r="BA76" s="240"/>
+      <c r="BB76" s="241"/>
     </row>
     <row r="77" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A77" s="250" t="b">
-        <v>0</v>
-      </c>
-      <c r="B77" s="252" t="s">
+      <c r="A77" s="248" t="b">
+        <v>0</v>
+      </c>
+      <c r="B77" s="250" t="s">
         <v>48</v>
       </c>
-      <c r="C77" s="112">
+      <c r="C77" s="111">
         <f>SUM(F77:BB77)</f>
         <v>1.5</v>
       </c>
-      <c r="D77" s="112">
+      <c r="D77" s="111">
         <f>SUM(F78:BB78)</f>
         <v>0</v>
       </c>
@@ -7565,8 +7592,8 @@
       <c r="BB77" s="40"/>
     </row>
     <row r="78" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A78" s="251"/>
-      <c r="B78" s="253"/>
+      <c r="A78" s="249"/>
+      <c r="B78" s="251"/>
       <c r="C78" s="102"/>
       <c r="D78" s="102"/>
       <c r="E78" s="106"/>
@@ -7621,21 +7648,21 @@
       <c r="BB78" s="29"/>
     </row>
     <row r="79" spans="1:54" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A79" s="254" t="b">
-        <v>0</v>
-      </c>
-      <c r="B79" s="255" t="s">
+      <c r="A79" s="252" t="b">
+        <v>0</v>
+      </c>
+      <c r="B79" s="253" t="s">
         <v>49</v>
       </c>
-      <c r="C79" s="112">
+      <c r="C79" s="111">
         <f>SUM(F79:BB79)</f>
         <v>1</v>
       </c>
-      <c r="D79" s="112">
+      <c r="D79" s="111">
         <f>SUM(F80:BB80)</f>
         <v>0</v>
       </c>
-      <c r="E79" s="113">
+      <c r="E79" s="112">
         <f t="shared" ref="E79:E83" si="5">(AVERAGE(C79,C80)-AVERAGE(D79,D80) )</f>
         <v>1</v>
       </c>
@@ -7692,8 +7719,8 @@
       <c r="BB79" s="26"/>
     </row>
     <row r="80" spans="1:54" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A80" s="251"/>
-      <c r="B80" s="253"/>
+      <c r="A80" s="249"/>
+      <c r="B80" s="251"/>
       <c r="C80" s="102"/>
       <c r="D80" s="102"/>
       <c r="E80" s="106"/>
@@ -7748,21 +7775,21 @@
       <c r="BB80" s="29"/>
     </row>
     <row r="81" spans="1:55" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A81" s="256" t="b">
-        <v>0</v>
-      </c>
-      <c r="B81" s="257" t="s">
+      <c r="A81" s="254" t="b">
+        <v>0</v>
+      </c>
+      <c r="B81" s="255" t="s">
         <v>52</v>
       </c>
-      <c r="C81" s="112">
+      <c r="C81" s="111">
         <f>SUM(F81:BB81)</f>
         <v>2.5</v>
       </c>
-      <c r="D81" s="112">
+      <c r="D81" s="111">
         <f>SUM(F82:BB82)</f>
         <v>0</v>
       </c>
-      <c r="E81" s="113">
+      <c r="E81" s="112">
         <f t="shared" si="5"/>
         <v>2.5</v>
       </c>
@@ -7821,8 +7848,8 @@
       <c r="BB81" s="32"/>
     </row>
     <row r="82" spans="1:55" ht="16" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A82" s="251"/>
-      <c r="B82" s="253"/>
+      <c r="A82" s="249"/>
+      <c r="B82" s="251"/>
       <c r="C82" s="102"/>
       <c r="D82" s="102"/>
       <c r="E82" s="106"/>
@@ -7877,21 +7904,21 @@
       <c r="BB82" s="29"/>
     </row>
     <row r="83" spans="1:55" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A83" s="254" t="b">
-        <v>0</v>
-      </c>
-      <c r="B83" s="255" t="s">
+      <c r="A83" s="252" t="b">
+        <v>0</v>
+      </c>
+      <c r="B83" s="253" t="s">
         <v>51</v>
       </c>
-      <c r="C83" s="112">
+      <c r="C83" s="111">
         <f>SUM(F83:BB83)</f>
         <v>5.5</v>
       </c>
-      <c r="D83" s="112">
+      <c r="D83" s="111">
         <f>SUM(F84:BB84)</f>
         <v>0</v>
       </c>
-      <c r="E83" s="113">
+      <c r="E83" s="112">
         <f t="shared" si="5"/>
         <v>5.5</v>
       </c>
@@ -7954,8 +7981,8 @@
       <c r="BB83" s="32"/>
     </row>
     <row r="84" spans="1:55" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A84" s="251"/>
-      <c r="B84" s="253"/>
+      <c r="A84" s="249"/>
+      <c r="B84" s="251"/>
       <c r="C84" s="102"/>
       <c r="D84" s="102"/>
       <c r="E84" s="106"/>
@@ -8010,21 +8037,21 @@
       <c r="BB84" s="29"/>
     </row>
     <row r="85" spans="1:55" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A85" s="254" t="b">
-        <v>0</v>
-      </c>
-      <c r="B85" s="268" t="s">
+      <c r="A85" s="252" t="b">
+        <v>0</v>
+      </c>
+      <c r="B85" s="266" t="s">
         <v>50</v>
       </c>
-      <c r="C85" s="112">
+      <c r="C85" s="111">
         <f>SUM(F85:BB85)</f>
         <v>0.5</v>
       </c>
-      <c r="D85" s="112">
+      <c r="D85" s="111">
         <f>SUM(F86:BB86)</f>
         <v>0</v>
       </c>
-      <c r="E85" s="113">
+      <c r="E85" s="112">
         <f>(AVERAGE(C85,C86)-AVERAGE(D85,D86) )</f>
         <v>0.5</v>
       </c>
@@ -8081,11 +8108,11 @@
       </c>
     </row>
     <row r="86" spans="1:55" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A86" s="256"/>
-      <c r="B86" s="269"/>
+      <c r="A86" s="254"/>
+      <c r="B86" s="267"/>
       <c r="C86" s="102"/>
       <c r="D86" s="102"/>
-      <c r="E86" s="145"/>
+      <c r="E86" s="143"/>
       <c r="F86" s="25"/>
       <c r="G86" s="58"/>
       <c r="H86" s="58"/>
@@ -8137,142 +8164,142 @@
       <c r="BB86" s="26"/>
     </row>
     <row r="87" spans="1:55" ht="15" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A87" s="270" t="s">
+      <c r="A87" s="268" t="s">
         <v>21</v>
       </c>
-      <c r="B87" s="271"/>
-      <c r="C87" s="274">
+      <c r="B87" s="269"/>
+      <c r="C87" s="272">
         <f>SUM(C89,C92)</f>
         <v>22</v>
       </c>
-      <c r="D87" s="274">
+      <c r="D87" s="272">
         <f>SUM(D89)</f>
         <v>2.5</v>
       </c>
-      <c r="E87" s="276">
+      <c r="E87" s="274">
         <f>(C87-D87)</f>
         <v>19.5</v>
       </c>
-      <c r="F87" s="258"/>
-      <c r="G87" s="259"/>
-      <c r="H87" s="259"/>
-      <c r="I87" s="259"/>
-      <c r="J87" s="259"/>
-      <c r="K87" s="259"/>
-      <c r="L87" s="259"/>
-      <c r="M87" s="259"/>
-      <c r="N87" s="259"/>
-      <c r="O87" s="259"/>
-      <c r="P87" s="259"/>
-      <c r="Q87" s="259"/>
-      <c r="R87" s="259"/>
-      <c r="S87" s="259"/>
-      <c r="T87" s="259"/>
-      <c r="U87" s="259"/>
-      <c r="V87" s="259"/>
-      <c r="W87" s="259"/>
-      <c r="X87" s="259"/>
-      <c r="Y87" s="259"/>
-      <c r="Z87" s="259"/>
-      <c r="AA87" s="259"/>
-      <c r="AB87" s="259"/>
-      <c r="AC87" s="259"/>
-      <c r="AD87" s="259"/>
-      <c r="AE87" s="259"/>
-      <c r="AF87" s="259"/>
-      <c r="AG87" s="259"/>
-      <c r="AH87" s="259"/>
-      <c r="AI87" s="259"/>
-      <c r="AJ87" s="259"/>
-      <c r="AK87" s="259"/>
-      <c r="AL87" s="259"/>
-      <c r="AM87" s="259"/>
-      <c r="AN87" s="259"/>
-      <c r="AO87" s="259"/>
-      <c r="AP87" s="259"/>
-      <c r="AQ87" s="259"/>
-      <c r="AR87" s="259"/>
-      <c r="AS87" s="259"/>
-      <c r="AT87" s="259"/>
-      <c r="AU87" s="259"/>
-      <c r="AV87" s="259"/>
-      <c r="AW87" s="259"/>
-      <c r="AX87" s="259"/>
-      <c r="AY87" s="259"/>
-      <c r="AZ87" s="259"/>
-      <c r="BA87" s="259"/>
-      <c r="BB87" s="260"/>
+      <c r="F87" s="256"/>
+      <c r="G87" s="257"/>
+      <c r="H87" s="257"/>
+      <c r="I87" s="257"/>
+      <c r="J87" s="257"/>
+      <c r="K87" s="257"/>
+      <c r="L87" s="257"/>
+      <c r="M87" s="257"/>
+      <c r="N87" s="257"/>
+      <c r="O87" s="257"/>
+      <c r="P87" s="257"/>
+      <c r="Q87" s="257"/>
+      <c r="R87" s="257"/>
+      <c r="S87" s="257"/>
+      <c r="T87" s="257"/>
+      <c r="U87" s="257"/>
+      <c r="V87" s="257"/>
+      <c r="W87" s="257"/>
+      <c r="X87" s="257"/>
+      <c r="Y87" s="257"/>
+      <c r="Z87" s="257"/>
+      <c r="AA87" s="257"/>
+      <c r="AB87" s="257"/>
+      <c r="AC87" s="257"/>
+      <c r="AD87" s="257"/>
+      <c r="AE87" s="257"/>
+      <c r="AF87" s="257"/>
+      <c r="AG87" s="257"/>
+      <c r="AH87" s="257"/>
+      <c r="AI87" s="257"/>
+      <c r="AJ87" s="257"/>
+      <c r="AK87" s="257"/>
+      <c r="AL87" s="257"/>
+      <c r="AM87" s="257"/>
+      <c r="AN87" s="257"/>
+      <c r="AO87" s="257"/>
+      <c r="AP87" s="257"/>
+      <c r="AQ87" s="257"/>
+      <c r="AR87" s="257"/>
+      <c r="AS87" s="257"/>
+      <c r="AT87" s="257"/>
+      <c r="AU87" s="257"/>
+      <c r="AV87" s="257"/>
+      <c r="AW87" s="257"/>
+      <c r="AX87" s="257"/>
+      <c r="AY87" s="257"/>
+      <c r="AZ87" s="257"/>
+      <c r="BA87" s="257"/>
+      <c r="BB87" s="258"/>
     </row>
     <row r="88" spans="1:55" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A88" s="272"/>
-      <c r="B88" s="273"/>
-      <c r="C88" s="275"/>
-      <c r="D88" s="275"/>
-      <c r="E88" s="277"/>
-      <c r="F88" s="261"/>
-      <c r="G88" s="262"/>
-      <c r="H88" s="262"/>
-      <c r="I88" s="262"/>
-      <c r="J88" s="262"/>
-      <c r="K88" s="262"/>
-      <c r="L88" s="262"/>
-      <c r="M88" s="262"/>
-      <c r="N88" s="262"/>
-      <c r="O88" s="262"/>
-      <c r="P88" s="262"/>
-      <c r="Q88" s="262"/>
-      <c r="R88" s="262"/>
-      <c r="S88" s="262"/>
-      <c r="T88" s="262"/>
-      <c r="U88" s="262"/>
-      <c r="V88" s="262"/>
-      <c r="W88" s="262"/>
-      <c r="X88" s="262"/>
-      <c r="Y88" s="262"/>
-      <c r="Z88" s="262"/>
-      <c r="AA88" s="262"/>
-      <c r="AB88" s="262"/>
-      <c r="AC88" s="262"/>
-      <c r="AD88" s="262"/>
-      <c r="AE88" s="262"/>
-      <c r="AF88" s="262"/>
-      <c r="AG88" s="262"/>
-      <c r="AH88" s="262"/>
-      <c r="AI88" s="262"/>
-      <c r="AJ88" s="262"/>
-      <c r="AK88" s="262"/>
-      <c r="AL88" s="262"/>
-      <c r="AM88" s="262"/>
-      <c r="AN88" s="262"/>
-      <c r="AO88" s="262"/>
-      <c r="AP88" s="262"/>
-      <c r="AQ88" s="262"/>
-      <c r="AR88" s="262"/>
-      <c r="AS88" s="262"/>
-      <c r="AT88" s="262"/>
-      <c r="AU88" s="262"/>
-      <c r="AV88" s="262"/>
-      <c r="AW88" s="262"/>
-      <c r="AX88" s="262"/>
-      <c r="AY88" s="262"/>
-      <c r="AZ88" s="262"/>
-      <c r="BA88" s="262"/>
-      <c r="BB88" s="263"/>
+      <c r="A88" s="270"/>
+      <c r="B88" s="271"/>
+      <c r="C88" s="273"/>
+      <c r="D88" s="273"/>
+      <c r="E88" s="275"/>
+      <c r="F88" s="259"/>
+      <c r="G88" s="260"/>
+      <c r="H88" s="260"/>
+      <c r="I88" s="260"/>
+      <c r="J88" s="260"/>
+      <c r="K88" s="260"/>
+      <c r="L88" s="260"/>
+      <c r="M88" s="260"/>
+      <c r="N88" s="260"/>
+      <c r="O88" s="260"/>
+      <c r="P88" s="260"/>
+      <c r="Q88" s="260"/>
+      <c r="R88" s="260"/>
+      <c r="S88" s="260"/>
+      <c r="T88" s="260"/>
+      <c r="U88" s="260"/>
+      <c r="V88" s="260"/>
+      <c r="W88" s="260"/>
+      <c r="X88" s="260"/>
+      <c r="Y88" s="260"/>
+      <c r="Z88" s="260"/>
+      <c r="AA88" s="260"/>
+      <c r="AB88" s="260"/>
+      <c r="AC88" s="260"/>
+      <c r="AD88" s="260"/>
+      <c r="AE88" s="260"/>
+      <c r="AF88" s="260"/>
+      <c r="AG88" s="260"/>
+      <c r="AH88" s="260"/>
+      <c r="AI88" s="260"/>
+      <c r="AJ88" s="260"/>
+      <c r="AK88" s="260"/>
+      <c r="AL88" s="260"/>
+      <c r="AM88" s="260"/>
+      <c r="AN88" s="260"/>
+      <c r="AO88" s="260"/>
+      <c r="AP88" s="260"/>
+      <c r="AQ88" s="260"/>
+      <c r="AR88" s="260"/>
+      <c r="AS88" s="260"/>
+      <c r="AT88" s="260"/>
+      <c r="AU88" s="260"/>
+      <c r="AV88" s="260"/>
+      <c r="AW88" s="260"/>
+      <c r="AX88" s="260"/>
+      <c r="AY88" s="260"/>
+      <c r="AZ88" s="260"/>
+      <c r="BA88" s="260"/>
+      <c r="BB88" s="261"/>
     </row>
     <row r="89" spans="1:55" x14ac:dyDescent="0.55000000000000004">
       <c r="A89" s="41"/>
-      <c r="B89" s="264" t="s">
-        <v>65</v>
-      </c>
-      <c r="C89" s="112">
+      <c r="B89" s="262" t="s">
+        <v>64</v>
+      </c>
+      <c r="C89" s="111">
         <f>SUM(F89:BB89)</f>
         <v>22</v>
       </c>
-      <c r="D89" s="112">
+      <c r="D89" s="111">
         <f>SUM(F90:BB90)</f>
         <v>2.5</v>
       </c>
-      <c r="E89" s="113">
+      <c r="E89" s="112">
         <f>(AVERAGE(C89,C90)-AVERAGE(D89,D90) )</f>
         <v>19.5</v>
       </c>
@@ -8308,7 +8335,7 @@
         <v>0.5</v>
       </c>
       <c r="S89" s="66">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="T89" s="67"/>
       <c r="U89" s="68"/>
@@ -8365,9 +8392,7 @@
       <c r="AP89" s="66">
         <v>0.5</v>
       </c>
-      <c r="AQ89" s="66">
-        <v>0.5</v>
-      </c>
+      <c r="AQ89" s="31"/>
       <c r="AR89" s="66">
         <v>0.5</v>
       </c>
@@ -8400,10 +8425,10 @@
     </row>
     <row r="90" spans="1:55" ht="14.7" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A90" s="42"/>
-      <c r="B90" s="265"/>
+      <c r="B90" s="263"/>
       <c r="C90" s="102"/>
       <c r="D90" s="102"/>
-      <c r="E90" s="145"/>
+      <c r="E90" s="143"/>
       <c r="F90" s="77">
         <v>1</v>
       </c>
@@ -8463,15 +8488,15 @@
       <c r="BC90" s="76"/>
     </row>
     <row r="91" spans="1:55" ht="15.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A91" s="280"/>
-      <c r="B91" s="281" t="s">
+      <c r="A91" s="278"/>
+      <c r="B91" s="279" t="s">
         <v>22</v>
       </c>
-      <c r="C91" s="283">
+      <c r="C91" s="281">
         <f>SUM((F91:BB91))</f>
         <v>1</v>
       </c>
-      <c r="D91" s="112"/>
+      <c r="D91" s="111"/>
       <c r="E91" s="101"/>
       <c r="F91" s="30"/>
       <c r="G91" s="31"/>
@@ -8527,11 +8552,11 @@
       <c r="BC91" s="76"/>
     </row>
     <row r="92" spans="1:55" ht="15.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A92" s="279"/>
-      <c r="B92" s="282"/>
-      <c r="C92" s="284"/>
-      <c r="D92" s="285"/>
-      <c r="E92" s="285"/>
+      <c r="A92" s="277"/>
+      <c r="B92" s="280"/>
+      <c r="C92" s="282"/>
+      <c r="D92" s="283"/>
+      <c r="E92" s="283"/>
       <c r="F92" s="27"/>
       <c r="G92" s="28"/>
       <c r="H92" s="28"/>
@@ -8592,61 +8617,61 @@
       </c>
       <c r="D93" s="47">
         <f>SUM(D21,D29,D41,D49,D67,D75,D87, D15,D6)</f>
-        <v>8</v>
+        <v>10.5</v>
       </c>
       <c r="E93" s="48">
         <f>SUM(E21,E29,E41,E49,E67,E75,E87,E6,E15)</f>
-        <v>72</v>
-      </c>
-      <c r="F93" s="266"/>
-      <c r="G93" s="267"/>
-      <c r="H93" s="267"/>
-      <c r="I93" s="267"/>
-      <c r="J93" s="267"/>
-      <c r="K93" s="267"/>
-      <c r="L93" s="267"/>
-      <c r="M93" s="267"/>
-      <c r="N93" s="267"/>
-      <c r="O93" s="267"/>
-      <c r="P93" s="267"/>
-      <c r="Q93" s="267"/>
-      <c r="R93" s="267"/>
-      <c r="S93" s="267"/>
-      <c r="T93" s="267"/>
-      <c r="U93" s="267"/>
-      <c r="V93" s="267"/>
-      <c r="W93" s="267"/>
-      <c r="X93" s="267"/>
-      <c r="Y93" s="267"/>
-      <c r="Z93" s="267"/>
-      <c r="AA93" s="267"/>
-      <c r="AB93" s="267"/>
-      <c r="AC93" s="267"/>
-      <c r="AD93" s="267"/>
-      <c r="AE93" s="267"/>
-      <c r="AF93" s="267"/>
-      <c r="AG93" s="267"/>
-      <c r="AH93" s="267"/>
-      <c r="AI93" s="267"/>
-      <c r="AJ93" s="267"/>
-      <c r="AK93" s="267"/>
-      <c r="AL93" s="267"/>
-      <c r="AM93" s="267"/>
-      <c r="AN93" s="267"/>
-      <c r="AO93" s="267"/>
-      <c r="AP93" s="267"/>
-      <c r="AQ93" s="267"/>
-      <c r="AR93" s="267"/>
-      <c r="AS93" s="267"/>
-      <c r="AT93" s="267"/>
-      <c r="AU93" s="267"/>
-      <c r="AV93" s="267"/>
-      <c r="AW93" s="267"/>
-      <c r="AX93" s="267"/>
-      <c r="AY93" s="267"/>
-      <c r="AZ93" s="267"/>
-      <c r="BA93" s="267"/>
-      <c r="BB93" s="267"/>
+        <v>69.5</v>
+      </c>
+      <c r="F93" s="264"/>
+      <c r="G93" s="265"/>
+      <c r="H93" s="265"/>
+      <c r="I93" s="265"/>
+      <c r="J93" s="265"/>
+      <c r="K93" s="265"/>
+      <c r="L93" s="265"/>
+      <c r="M93" s="265"/>
+      <c r="N93" s="265"/>
+      <c r="O93" s="265"/>
+      <c r="P93" s="265"/>
+      <c r="Q93" s="265"/>
+      <c r="R93" s="265"/>
+      <c r="S93" s="265"/>
+      <c r="T93" s="265"/>
+      <c r="U93" s="265"/>
+      <c r="V93" s="265"/>
+      <c r="W93" s="265"/>
+      <c r="X93" s="265"/>
+      <c r="Y93" s="265"/>
+      <c r="Z93" s="265"/>
+      <c r="AA93" s="265"/>
+      <c r="AB93" s="265"/>
+      <c r="AC93" s="265"/>
+      <c r="AD93" s="265"/>
+      <c r="AE93" s="265"/>
+      <c r="AF93" s="265"/>
+      <c r="AG93" s="265"/>
+      <c r="AH93" s="265"/>
+      <c r="AI93" s="265"/>
+      <c r="AJ93" s="265"/>
+      <c r="AK93" s="265"/>
+      <c r="AL93" s="265"/>
+      <c r="AM93" s="265"/>
+      <c r="AN93" s="265"/>
+      <c r="AO93" s="265"/>
+      <c r="AP93" s="265"/>
+      <c r="AQ93" s="265"/>
+      <c r="AR93" s="265"/>
+      <c r="AS93" s="265"/>
+      <c r="AT93" s="265"/>
+      <c r="AU93" s="265"/>
+      <c r="AV93" s="265"/>
+      <c r="AW93" s="265"/>
+      <c r="AX93" s="265"/>
+      <c r="AY93" s="265"/>
+      <c r="AZ93" s="265"/>
+      <c r="BA93" s="265"/>
+      <c r="BB93" s="265"/>
     </row>
     <row r="94" spans="1:55" ht="75.599999999999994" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="C94" s="49" t="s">

</xml_diff>